<commit_message>
feat: release v2.16.0 with central controller checklist, compact UI, auto-hiding empty columns, RA p-board quotation, and pipe sizing formatting
</commit_message>
<xml_diff>
--- a/backend/product_database/EQUIPMENT_Data.xlsx
+++ b/backend/product_database/EQUIPMENT_Data.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flitt\.gemini\antigravity\scratch\ac-selection-system\backend\product_database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13BF260E-39DE-446D-9F65-2A53F1EA4FB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9720F7D1-E31A-4D22-AF43-EAB288AFF7AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="48" windowWidth="11832" windowHeight="12240" xr2:uid="{B9AE4098-F0A1-4C76-B9D5-37F1BE2208A4}"/>
+    <workbookView xWindow="960" yWindow="720" windowWidth="22080" windowHeight="12240" activeTab="1" xr2:uid="{B9AE4098-F0A1-4C76-B9D5-37F1BE2208A4}"/>
   </bookViews>
   <sheets>
     <sheet name="indoor_units" sheetId="1" r:id="rId1"/>
-    <sheet name="outdoor_units" sheetId="2" r:id="rId2"/>
-    <sheet name="indoor_units_SA only" sheetId="3" r:id="rId3"/>
-    <sheet name="outdoor_units_SA only" sheetId="4" r:id="rId4"/>
+    <sheet name="controller" sheetId="5" r:id="rId2"/>
+    <sheet name="outdoor_units" sheetId="2" r:id="rId3"/>
+    <sheet name="indoor_units_SA only" sheetId="3" r:id="rId4"/>
+    <sheet name="outdoor_units_SA only" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3544" uniqueCount="569">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3765" uniqueCount="621">
   <si>
     <t>資料型態</t>
   </si>
@@ -2174,6 +2175,214 @@
     <t>無線遙控器</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>2MXP85ZVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>395×930×350</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BRC1E63R</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BRC4C65</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BRC4C62-9</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BRC7M634F</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BRC7M675</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BRC7EA63W9</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BRC7M530W</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BRC7M65</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>集中控制器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DCS301BA61</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>集中ON-OFF控制器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>中央集中控制器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DCS302CA61</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DCS303A61</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DST301BA61</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>家用集中控制器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>預定時程控制器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DTP401A61</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DTP401A63</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>中央集控外接監控基板</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DCS302A52</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>STC集中控制器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>STC集中控制器電源</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DCM601B51</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ITM</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DGE601A52</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ITM擴充卡1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DGE601A53</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ITM擴充卡插槽</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DCM009A51</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DCM007A51</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ITM WEB網路</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>網路接伶俐</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DTA116A51</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Modbus 介面</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BACnet 介面</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ITM BACnet協定軟體</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DMS502B51</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DAM411B51</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BACnet 擴充組</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DCPA01</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>伶俐用轉接器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DCPF01</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>伶俐智控管理器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>型號</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>中文名稱</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>報價</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>低階</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>高階</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>備註</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -2181,8 +2390,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="176" formatCode="0.0_ "/>
-    <numFmt numFmtId="178" formatCode="#,##0_ "/>
-    <numFmt numFmtId="179" formatCode="#,##0_);[Red]\(#,##0\)"/>
+    <numFmt numFmtId="177" formatCode="#,##0_ "/>
+    <numFmt numFmtId="178" formatCode="#,##0_);[Red]\(#,##0\)"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -2260,7 +2469,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2270,6 +2479,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2381,7 +2596,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2523,34 +2738,55 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="178" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="178" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="179" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="178" fontId="3" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2875,7 +3111,9 @@
     <col min="3" max="3" width="14.6640625" style="6" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="41.44140625" style="2" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="10.6640625" style="6" customWidth="1"/>
-    <col min="6" max="193" width="10.6640625" style="2" customWidth="1"/>
+    <col min="6" max="87" width="10.6640625" style="2" customWidth="1"/>
+    <col min="88" max="88" width="12.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="89" max="193" width="10.6640625" style="2" customWidth="1"/>
     <col min="194" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
@@ -4829,7 +5067,7 @@
       </c>
       <c r="GL4" s="5"/>
     </row>
-    <row r="5" spans="1:194" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:194" ht="16.2" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="32" t="s">
         <v>46</v>
       </c>
@@ -5411,7 +5649,7 @@
       </c>
       <c r="GL5" s="5"/>
     </row>
-    <row r="6" spans="1:194" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:194" ht="16.2" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="32" t="s">
         <v>474</v>
       </c>
@@ -5993,7 +6231,7 @@
       </c>
       <c r="GL6" s="5"/>
     </row>
-    <row r="7" spans="1:194" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:194" ht="24.6" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="32" t="s">
         <v>475</v>
       </c>
@@ -6575,7 +6813,7 @@
       </c>
       <c r="GL7" s="5"/>
     </row>
-    <row r="8" spans="1:194" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:194" ht="16.2" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="32" t="s">
         <v>47</v>
       </c>
@@ -7157,7 +7395,7 @@
       </c>
       <c r="GL8" s="5"/>
     </row>
-    <row r="9" spans="1:194" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:194" ht="16.2" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="32" t="s">
         <v>59</v>
       </c>
@@ -7739,7 +7977,7 @@
       </c>
       <c r="GL9" s="5"/>
     </row>
-    <row r="10" spans="1:194" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:194" ht="24.6" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="32" t="s">
         <v>58</v>
       </c>
@@ -8321,7 +8559,7 @@
       </c>
       <c r="GL10" s="5"/>
     </row>
-    <row r="11" spans="1:194" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:194" ht="24.6" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="38" t="s">
         <v>51</v>
       </c>
@@ -8903,7 +9141,7 @@
       </c>
       <c r="GL11" s="5"/>
     </row>
-    <row r="12" spans="1:194" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:194" ht="24.6" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="39" t="s">
         <v>61</v>
       </c>
@@ -9485,7 +9723,7 @@
       </c>
       <c r="GL12" s="9"/>
     </row>
-    <row r="13" spans="1:194" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:194" ht="16.2" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="40" t="s">
         <v>543</v>
       </c>
@@ -9686,7 +9924,7 @@
       <c r="GJ13" s="40"/>
       <c r="GK13" s="40"/>
     </row>
-    <row r="14" spans="1:194" customFormat="1" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:194" customFormat="1" ht="16.8" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="39" t="s">
         <v>540</v>
       </c>
@@ -10053,7 +10291,7 @@
       <c r="GJ14" s="44"/>
       <c r="GK14" s="44"/>
     </row>
-    <row r="15" spans="1:194" customFormat="1" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:194" customFormat="1" ht="16.8" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="39" t="s">
         <v>544</v>
       </c>
@@ -10418,7 +10656,7 @@
       <c r="GJ15" s="44"/>
       <c r="GK15" s="44"/>
     </row>
-    <row r="16" spans="1:194" customFormat="1" ht="25.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:194" customFormat="1" ht="25.8" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="39" t="s">
         <v>541</v>
       </c>
@@ -10783,7 +11021,7 @@
       <c r="GJ16" s="44"/>
       <c r="GK16" s="44"/>
     </row>
-    <row r="17" spans="1:13" s="52" customFormat="1" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:193" s="52" customFormat="1" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="52" t="s">
         <v>562</v>
       </c>
@@ -10796,42 +11034,1006 @@
       <c r="D17" s="54" t="s">
         <v>563</v>
       </c>
-      <c r="E17" s="55">
+      <c r="E17" s="57">
         <v>0</v>
       </c>
-      <c r="F17" s="55">
+      <c r="F17" s="57">
         <v>0</v>
       </c>
-      <c r="G17" s="55">
+      <c r="G17" s="57">
         <v>0</v>
       </c>
-      <c r="H17" s="55">
+      <c r="H17" s="57">
         <v>0</v>
       </c>
-      <c r="I17" s="55">
+      <c r="I17" s="57">
         <v>0</v>
       </c>
-      <c r="J17" s="55">
+      <c r="J17" s="57">
         <v>0</v>
       </c>
-      <c r="K17" s="55">
+      <c r="K17" s="57">
         <v>0</v>
       </c>
-      <c r="L17" s="55">
+      <c r="L17" s="57">
         <v>0</v>
       </c>
-      <c r="M17" s="55">
+      <c r="M17" s="57">
         <v>0</v>
       </c>
+      <c r="N17" s="58">
+        <v>17280</v>
+      </c>
+      <c r="O17" s="58">
+        <v>19080</v>
+      </c>
+      <c r="P17" s="58">
+        <v>22080</v>
+      </c>
+      <c r="Q17" s="58">
+        <v>24380</v>
+      </c>
+      <c r="R17" s="58">
+        <v>27720</v>
+      </c>
+      <c r="S17" s="58">
+        <v>30220</v>
+      </c>
+      <c r="T17" s="58">
+        <v>33520</v>
+      </c>
+      <c r="U17" s="58">
+        <v>18180</v>
+      </c>
+      <c r="V17" s="58">
+        <v>19980</v>
+      </c>
+      <c r="W17" s="58">
+        <v>23680</v>
+      </c>
+      <c r="X17" s="58">
+        <v>24780</v>
+      </c>
+      <c r="Y17" s="58">
+        <v>27920</v>
+      </c>
+      <c r="Z17" s="58">
+        <v>30220</v>
+      </c>
+      <c r="AA17" s="58">
+        <v>32720</v>
+      </c>
+      <c r="AB17" s="58">
+        <v>37520</v>
+      </c>
+      <c r="AC17" s="58">
+        <v>41520</v>
+      </c>
+      <c r="AD17" s="58"/>
+      <c r="AE17" s="58"/>
+      <c r="AF17" s="58"/>
+      <c r="AG17" s="58"/>
+      <c r="AH17" s="58"/>
+      <c r="AI17" s="58"/>
+      <c r="AJ17" s="58"/>
+      <c r="AK17" s="58">
+        <v>14080</v>
+      </c>
+      <c r="AL17" s="58">
+        <v>16180</v>
+      </c>
+      <c r="AM17" s="58">
+        <v>17480</v>
+      </c>
+      <c r="AN17" s="58">
+        <v>19980</v>
+      </c>
+      <c r="AO17" s="58">
+        <v>23820</v>
+      </c>
+      <c r="AP17" s="58">
+        <v>27220</v>
+      </c>
+      <c r="AQ17" s="58">
+        <v>30220</v>
+      </c>
+      <c r="AR17" s="58"/>
+      <c r="AS17" s="58"/>
+      <c r="AT17" s="58"/>
+      <c r="AU17" s="58"/>
+      <c r="AV17" s="58"/>
+      <c r="AW17" s="58"/>
+      <c r="AX17" s="58"/>
+      <c r="AY17" s="58">
+        <v>12980</v>
+      </c>
+      <c r="AZ17" s="58">
+        <v>14080</v>
+      </c>
+      <c r="BA17" s="58">
+        <v>15380</v>
+      </c>
+      <c r="BB17" s="58">
+        <v>18280</v>
+      </c>
+      <c r="BC17" s="58">
+        <v>21520</v>
+      </c>
+      <c r="BD17" s="58">
+        <v>24320</v>
+      </c>
+      <c r="BE17" s="58">
+        <v>27320</v>
+      </c>
+      <c r="BF17" s="58">
+        <v>16680</v>
+      </c>
+      <c r="BG17" s="58">
+        <v>17980</v>
+      </c>
+      <c r="BH17" s="58">
+        <v>20280</v>
+      </c>
+      <c r="BI17" s="58">
+        <v>22080</v>
+      </c>
+      <c r="BJ17" s="58">
+        <v>25020</v>
+      </c>
+      <c r="BK17" s="58">
+        <v>25620</v>
+      </c>
+      <c r="BL17" s="58">
+        <v>27720</v>
+      </c>
+      <c r="BM17" s="58">
+        <v>17280</v>
+      </c>
+      <c r="BN17" s="58">
+        <v>19080</v>
+      </c>
+      <c r="BO17" s="58">
+        <v>22080</v>
+      </c>
+      <c r="BP17" s="58">
+        <v>24380</v>
+      </c>
+      <c r="BQ17" s="58">
+        <v>27720</v>
+      </c>
+      <c r="BR17" s="58">
+        <v>30220</v>
+      </c>
+      <c r="BS17" s="58">
+        <v>33520</v>
+      </c>
+      <c r="BT17" s="58">
+        <v>34100</v>
+      </c>
+      <c r="BU17" s="58">
+        <v>38100</v>
+      </c>
+      <c r="BV17" s="58">
+        <v>16680</v>
+      </c>
+      <c r="BW17" s="58">
+        <v>17980</v>
+      </c>
+      <c r="BX17" s="58">
+        <v>20280</v>
+      </c>
+      <c r="BY17" s="58">
+        <v>22080</v>
+      </c>
+      <c r="BZ17" s="58">
+        <v>25020</v>
+      </c>
+      <c r="CA17" s="58">
+        <v>25620</v>
+      </c>
+      <c r="CB17" s="58">
+        <v>27720</v>
+      </c>
+      <c r="CC17" s="58">
+        <v>12980</v>
+      </c>
+      <c r="CD17" s="58">
+        <v>14080</v>
+      </c>
+      <c r="CE17" s="58">
+        <v>15380</v>
+      </c>
+      <c r="CF17" s="58">
+        <v>18280</v>
+      </c>
+      <c r="CG17" s="58">
+        <v>21520</v>
+      </c>
+      <c r="CH17" s="58">
+        <v>24320</v>
+      </c>
+      <c r="CI17" s="58">
+        <v>27320</v>
+      </c>
+      <c r="CJ17" s="58">
+        <v>26200</v>
+      </c>
+      <c r="CK17" s="58">
+        <v>27200</v>
+      </c>
+      <c r="CL17" s="58">
+        <v>28700</v>
+      </c>
+      <c r="CM17" s="58">
+        <v>30600</v>
+      </c>
+      <c r="CN17" s="58">
+        <v>32800</v>
+      </c>
+      <c r="CO17" s="58">
+        <v>35200</v>
+      </c>
+      <c r="CP17" s="58">
+        <v>29000</v>
+      </c>
+      <c r="CQ17" s="58">
+        <v>29900</v>
+      </c>
+      <c r="CR17" s="58">
+        <v>31500</v>
+      </c>
+      <c r="CS17" s="58">
+        <v>33400</v>
+      </c>
+      <c r="CT17" s="58">
+        <v>35700</v>
+      </c>
+      <c r="CU17" s="58">
+        <v>38100</v>
+      </c>
+      <c r="CV17" s="58">
+        <v>34800</v>
+      </c>
+      <c r="CW17" s="58">
+        <v>36100</v>
+      </c>
+      <c r="CX17" s="58">
+        <v>37200</v>
+      </c>
+      <c r="CY17" s="58">
+        <v>39000</v>
+      </c>
+      <c r="CZ17" s="58">
+        <v>40100</v>
+      </c>
+      <c r="DA17" s="58">
+        <v>43700</v>
+      </c>
+      <c r="DB17" s="58">
+        <v>48300</v>
+      </c>
+      <c r="DC17" s="58">
+        <v>51200</v>
+      </c>
+      <c r="DD17" s="58">
+        <v>53800</v>
+      </c>
+      <c r="DE17" s="58">
+        <v>62700</v>
+      </c>
+      <c r="DF17" s="58">
+        <v>36000</v>
+      </c>
+      <c r="DG17" s="58">
+        <v>37100</v>
+      </c>
+      <c r="DH17" s="58">
+        <v>38300</v>
+      </c>
+      <c r="DI17" s="58">
+        <v>40100</v>
+      </c>
+      <c r="DJ17" s="58">
+        <v>41100</v>
+      </c>
+      <c r="DK17" s="58">
+        <v>44700</v>
+      </c>
+      <c r="DL17" s="58">
+        <v>49300</v>
+      </c>
+      <c r="DM17" s="58">
+        <v>52300</v>
+      </c>
+      <c r="DN17" s="58">
+        <v>54800</v>
+      </c>
+      <c r="DO17" s="58">
+        <v>63800</v>
+      </c>
+      <c r="DP17" s="58">
+        <v>92800</v>
+      </c>
+      <c r="DQ17" s="58">
+        <v>98000</v>
+      </c>
+      <c r="DR17" s="58">
+        <v>110000</v>
+      </c>
+      <c r="DS17" s="58">
+        <v>116000</v>
+      </c>
+      <c r="DT17" s="58">
+        <v>108100</v>
+      </c>
+      <c r="DU17" s="58">
+        <v>129800</v>
+      </c>
+      <c r="DV17" s="58">
+        <v>140900</v>
+      </c>
+      <c r="DW17" s="58">
+        <v>57100</v>
+      </c>
+      <c r="DX17" s="58">
+        <v>79500</v>
+      </c>
+      <c r="DY17" s="58">
+        <v>113200</v>
+      </c>
+      <c r="DZ17" s="58">
+        <v>120300</v>
+      </c>
+      <c r="EA17" s="58">
+        <v>105000</v>
+      </c>
+      <c r="EB17" s="58">
+        <v>40000</v>
+      </c>
+      <c r="EC17" s="58">
+        <v>41400</v>
+      </c>
+      <c r="ED17" s="58">
+        <v>43100</v>
+      </c>
+      <c r="EE17" s="58">
+        <v>44300</v>
+      </c>
+      <c r="EF17" s="58">
+        <v>45400</v>
+      </c>
+      <c r="EG17" s="58">
+        <v>50000</v>
+      </c>
+      <c r="EH17" s="58">
+        <v>52900</v>
+      </c>
+      <c r="EI17" s="58">
+        <v>55500</v>
+      </c>
+      <c r="EJ17" s="58">
+        <v>64400</v>
+      </c>
+      <c r="EK17" s="58">
+        <v>43200</v>
+      </c>
+      <c r="EL17" s="58">
+        <v>45300</v>
+      </c>
+      <c r="EM17" s="58">
+        <v>47700</v>
+      </c>
+      <c r="EN17" s="58">
+        <v>48400</v>
+      </c>
+      <c r="EO17" s="58">
+        <v>49100</v>
+      </c>
+      <c r="EP17" s="58">
+        <v>53100</v>
+      </c>
+      <c r="EQ17" s="58">
+        <v>56300</v>
+      </c>
+      <c r="ER17" s="58">
+        <v>59500</v>
+      </c>
+      <c r="ES17" s="58">
+        <v>69500</v>
+      </c>
+      <c r="ET17" s="58">
+        <v>34300</v>
+      </c>
+      <c r="EU17" s="58">
+        <v>35400</v>
+      </c>
+      <c r="EV17" s="58">
+        <v>36500</v>
+      </c>
+      <c r="EW17" s="58">
+        <v>36800</v>
+      </c>
+      <c r="EX17" s="58">
+        <v>37000</v>
+      </c>
+      <c r="EY17" s="58">
+        <v>42100</v>
+      </c>
+      <c r="EZ17" s="58">
+        <v>45300</v>
+      </c>
+      <c r="FA17" s="58">
+        <v>51300</v>
+      </c>
+      <c r="FB17" s="58">
+        <v>59800</v>
+      </c>
+      <c r="FC17" s="58">
+        <v>185000</v>
+      </c>
+      <c r="FD17" s="61" t="s">
+        <v>37</v>
+      </c>
+      <c r="FE17" s="61" t="s">
+        <v>37</v>
+      </c>
+      <c r="FF17" s="58">
+        <v>34500</v>
+      </c>
+      <c r="FG17" s="58">
+        <v>38500</v>
+      </c>
+      <c r="FH17" s="58">
+        <v>39900</v>
+      </c>
+      <c r="FI17" s="58">
+        <v>41100</v>
+      </c>
+      <c r="FJ17" s="58">
+        <v>42300</v>
+      </c>
+      <c r="FK17" s="58">
+        <v>42000</v>
+      </c>
+      <c r="FL17" s="58">
+        <v>44200</v>
+      </c>
+      <c r="FM17" s="58">
+        <v>45800</v>
+      </c>
+      <c r="FN17" s="58">
+        <v>46900</v>
+      </c>
+      <c r="FO17" s="58">
+        <v>49800</v>
+      </c>
+      <c r="FP17" s="58">
+        <v>54800</v>
+      </c>
+      <c r="FQ17" s="58">
+        <v>61300</v>
+      </c>
+      <c r="FR17" s="58">
+        <v>66800</v>
+      </c>
+      <c r="FS17" s="58"/>
+      <c r="FT17" s="58"/>
+      <c r="FU17" s="58"/>
+      <c r="FV17" s="58"/>
+      <c r="FW17" s="58"/>
+      <c r="FX17" s="58"/>
+      <c r="FY17" s="58"/>
+      <c r="FZ17" s="58"/>
+      <c r="GA17" s="58"/>
+      <c r="GB17" s="58"/>
+      <c r="GC17" s="58"/>
+      <c r="GD17" s="58"/>
+      <c r="GE17" s="58"/>
+      <c r="GF17" s="58"/>
+      <c r="GG17" s="58"/>
+      <c r="GH17" s="58"/>
+      <c r="GI17" s="58"/>
+      <c r="GJ17" s="58"/>
+      <c r="GK17" s="58"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A18" s="24" t="s">
+    <row r="18" spans="1:193" s="40" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+      <c r="A18" s="59" t="s">
         <v>567</v>
       </c>
+      <c r="C18" s="41"/>
+      <c r="E18" s="41"/>
+      <c r="CJ18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="CK18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="CL18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="CM18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="CN18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="CO18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="CP18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="CQ18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="CR18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="CS18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="CT18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="CU18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="CV18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="CW18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="CX18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="CY18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="CZ18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DA18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DB18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DC18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DD18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DE18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DF18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DG18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DH18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DI18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DJ18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DK18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DL18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DM18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DN18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DO18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DP18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DQ18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DR18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DS18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DT18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DU18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DV18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DW18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DX18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DY18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="DZ18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EA18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EB18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EC18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="ED18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EE18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EF18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EG18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EH18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EI18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EJ18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EK18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EL18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EM18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EN18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EO18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EP18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EQ18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="ER18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="ES18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="ET18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EU18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EV18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EW18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EX18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EY18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="EZ18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="FA18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="FB18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="FC18" s="60" t="s">
+        <v>37</v>
+      </c>
+      <c r="FF18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="FG18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="FH18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="FI18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="FJ18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="FK18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="FL18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="FM18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="FN18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="FO18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="FP18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="FQ18" s="40" t="s">
+        <v>571</v>
+      </c>
+      <c r="FR18" s="40" t="s">
+        <v>571</v>
+      </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A19" s="24" t="s">
+    <row r="19" spans="1:193" s="40" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+      <c r="A19" s="59" t="s">
         <v>568</v>
+      </c>
+      <c r="C19" s="41"/>
+      <c r="E19" s="41"/>
+      <c r="CJ19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="CK19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="CL19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="CM19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="CN19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="CO19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="CP19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="CQ19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="CR19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="CS19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="CT19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="CU19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="CV19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="CW19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="CX19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="CY19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="CZ19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="DA19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="DB19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="DC19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="DD19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="DE19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="DF19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="DG19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="DH19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="DI19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="DJ19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="DK19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="DL19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="DM19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="DN19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="DO19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="DP19" s="40" t="s">
+        <v>573</v>
+      </c>
+      <c r="DQ19" s="40" t="s">
+        <v>573</v>
+      </c>
+      <c r="DR19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="DS19" s="40" t="s">
+        <v>572</v>
+      </c>
+      <c r="EB19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="EC19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="ED19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="EE19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="EF19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="EG19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="EH19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="EI19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="EJ19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="EK19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="EL19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="EM19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="EN19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="EO19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="EP19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="EQ19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="ER19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="ES19" s="40" t="s">
+        <v>574</v>
+      </c>
+      <c r="ET19" s="40" t="s">
+        <v>575</v>
+      </c>
+      <c r="EU19" s="40" t="s">
+        <v>575</v>
+      </c>
+      <c r="EV19" s="40" t="s">
+        <v>575</v>
+      </c>
+      <c r="EW19" s="40" t="s">
+        <v>575</v>
+      </c>
+      <c r="EX19" s="40" t="s">
+        <v>575</v>
+      </c>
+      <c r="EY19" s="40" t="s">
+        <v>575</v>
+      </c>
+      <c r="EZ19" s="40" t="s">
+        <v>576</v>
+      </c>
+      <c r="FA19" s="40" t="s">
+        <v>576</v>
+      </c>
+      <c r="FB19" s="40" t="s">
+        <v>576</v>
+      </c>
+      <c r="FC19" s="60" t="s">
+        <v>37</v>
+      </c>
+      <c r="FF19" s="40" t="s">
+        <v>577</v>
+      </c>
+      <c r="FG19" s="40" t="s">
+        <v>577</v>
+      </c>
+      <c r="FH19" s="40" t="s">
+        <v>577</v>
+      </c>
+      <c r="FI19" s="40" t="s">
+        <v>577</v>
+      </c>
+      <c r="FJ19" s="40" t="s">
+        <v>577</v>
+      </c>
+      <c r="FK19" s="40" t="s">
+        <v>578</v>
+      </c>
+      <c r="FL19" s="40" t="s">
+        <v>578</v>
+      </c>
+      <c r="FM19" s="40" t="s">
+        <v>578</v>
+      </c>
+      <c r="FN19" s="40" t="s">
+        <v>578</v>
+      </c>
+      <c r="FO19" s="40" t="s">
+        <v>578</v>
+      </c>
+      <c r="FP19" s="40" t="s">
+        <v>578</v>
+      </c>
+      <c r="FQ19" s="40" t="s">
+        <v>578</v>
+      </c>
+      <c r="FR19" s="40" t="s">
+        <v>578</v>
       </c>
     </row>
   </sheetData>
@@ -10842,18 +12044,269 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F00506A-09F5-4009-80F2-281B4A4C3425}">
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>615</v>
+      </c>
+      <c r="B2" t="s">
+        <v>616</v>
+      </c>
+      <c r="C2" t="s">
+        <v>617</v>
+      </c>
+      <c r="D2" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="62" t="s">
+        <v>580</v>
+      </c>
+      <c r="B3" s="62" t="s">
+        <v>581</v>
+      </c>
+      <c r="C3">
+        <v>11800</v>
+      </c>
+      <c r="D3" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="62" t="s">
+        <v>583</v>
+      </c>
+      <c r="B4" s="62" t="s">
+        <v>582</v>
+      </c>
+      <c r="C4">
+        <v>11700</v>
+      </c>
+      <c r="D4" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>591</v>
+      </c>
+      <c r="B5" t="s">
+        <v>590</v>
+      </c>
+      <c r="C5">
+        <v>4700</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="62" t="s">
+        <v>584</v>
+      </c>
+      <c r="B6" s="62" t="s">
+        <v>586</v>
+      </c>
+      <c r="C6">
+        <v>22800</v>
+      </c>
+      <c r="D6" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>585</v>
+      </c>
+      <c r="B7" t="s">
+        <v>587</v>
+      </c>
+      <c r="C7">
+        <v>7350</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="62" t="s">
+        <v>588</v>
+      </c>
+      <c r="B8" s="62" t="s">
+        <v>592</v>
+      </c>
+      <c r="C8">
+        <v>25000</v>
+      </c>
+      <c r="D8" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>589</v>
+      </c>
+      <c r="B9" t="s">
+        <v>593</v>
+      </c>
+      <c r="C9">
+        <v>2800</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="62" t="s">
+        <v>594</v>
+      </c>
+      <c r="B10" s="62" t="s">
+        <v>595</v>
+      </c>
+      <c r="C10">
+        <v>108200</v>
+      </c>
+      <c r="D10" t="s">
+        <v>619</v>
+      </c>
+      <c r="F10" s="63"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>596</v>
+      </c>
+      <c r="B11" t="s">
+        <v>597</v>
+      </c>
+      <c r="C11">
+        <v>28600</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>598</v>
+      </c>
+      <c r="B12" t="s">
+        <v>599</v>
+      </c>
+      <c r="C12">
+        <v>19400</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>601</v>
+      </c>
+      <c r="B13" t="s">
+        <v>602</v>
+      </c>
+      <c r="C13">
+        <v>19400</v>
+      </c>
+      <c r="D13" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>600</v>
+      </c>
+      <c r="B14" t="s">
+        <v>607</v>
+      </c>
+      <c r="C14">
+        <v>27500</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="62" t="s">
+        <v>604</v>
+      </c>
+      <c r="B15" s="62" t="s">
+        <v>605</v>
+      </c>
+      <c r="C15">
+        <v>11500</v>
+      </c>
+      <c r="D15" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="62" t="s">
+        <v>608</v>
+      </c>
+      <c r="B16" s="62" t="s">
+        <v>606</v>
+      </c>
+      <c r="C16">
+        <v>83600</v>
+      </c>
+      <c r="D16" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>609</v>
+      </c>
+      <c r="B17" t="s">
+        <v>610</v>
+      </c>
+      <c r="C17">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="62" t="s">
+        <v>611</v>
+      </c>
+      <c r="B18" s="62" t="s">
+        <v>612</v>
+      </c>
+      <c r="C18">
+        <v>9200</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="62" t="s">
+        <v>613</v>
+      </c>
+      <c r="B19" s="62" t="s">
+        <v>614</v>
+      </c>
+      <c r="C19">
+        <v>34700</v>
+      </c>
+      <c r="D19" t="s">
+        <v>619</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14518F8B-544C-42CB-BD27-24B9976359F4}">
-  <dimension ref="A1:FG15"/>
+  <dimension ref="A1:FH15"/>
   <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.44140625" customWidth="1"/>
     <col min="2" max="2" width="13.44140625" customWidth="1"/>
     <col min="3" max="3" width="16.44140625" style="7" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="34.44140625" hidden="1" customWidth="1"/>
-    <col min="5" max="130" width="14.6640625" customWidth="1"/>
+    <col min="5" max="131" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:163" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:164" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -10867,7 +12320,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:163" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:164" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>41</v>
       </c>
@@ -11055,7 +12508,7 @@
         <v>34</v>
       </c>
       <c r="BK2" s="5" t="s">
-        <v>133</v>
+        <v>34</v>
       </c>
       <c r="BL2" s="5" t="s">
         <v>133</v>
@@ -11258,7 +12711,9 @@
       <c r="DZ2" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="EA2" s="5"/>
+      <c r="EA2" s="5" t="s">
+        <v>133</v>
+      </c>
       <c r="EB2" s="5"/>
       <c r="EC2" s="5"/>
       <c r="ED2" s="5"/>
@@ -11291,8 +12746,9 @@
       <c r="FE2" s="5"/>
       <c r="FF2" s="5"/>
       <c r="FG2" s="5"/>
+      <c r="FH2" s="5"/>
     </row>
-    <row r="3" spans="1:163" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:164" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>44</v>
       </c>
@@ -11480,10 +12936,10 @@
         <v>476</v>
       </c>
       <c r="BK3" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="BL3" s="5" t="s">
         <v>128</v>
-      </c>
-      <c r="BL3" s="5" t="s">
-        <v>130</v>
       </c>
       <c r="BM3" s="5" t="s">
         <v>130</v>
@@ -11498,13 +12954,13 @@
         <v>130</v>
       </c>
       <c r="BQ3" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="BR3" s="5" t="s">
         <v>131</v>
       </c>
       <c r="BS3" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="BT3" s="5" t="s">
         <v>132</v>
@@ -11513,7 +12969,7 @@
         <v>132</v>
       </c>
       <c r="BV3" s="5" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
       <c r="BW3" s="5" t="s">
         <v>146</v>
@@ -11522,7 +12978,7 @@
         <v>146</v>
       </c>
       <c r="BY3" s="5" t="s">
-        <v>190</v>
+        <v>146</v>
       </c>
       <c r="BZ3" s="5" t="s">
         <v>190</v>
@@ -11603,7 +13059,7 @@
         <v>190</v>
       </c>
       <c r="CZ3" s="5" t="s">
-        <v>42</v>
+        <v>190</v>
       </c>
       <c r="DA3" s="5" t="s">
         <v>42</v>
@@ -11683,7 +13139,9 @@
       <c r="DZ3" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="EA3" s="5"/>
+      <c r="EA3" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="EB3" s="5"/>
       <c r="EC3" s="5"/>
       <c r="ED3" s="5"/>
@@ -11716,8 +13174,9 @@
       <c r="FE3" s="5"/>
       <c r="FF3" s="5"/>
       <c r="FG3" s="5"/>
+      <c r="FH3" s="5"/>
     </row>
-    <row r="4" spans="1:163" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:164" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>52</v>
       </c>
@@ -11905,210 +13364,212 @@
         <v>109</v>
       </c>
       <c r="BK4" s="5" t="s">
+        <v>569</v>
+      </c>
+      <c r="BL4" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="BL4" s="5" t="s">
+      <c r="BM4" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="BM4" s="5" t="s">
+      <c r="BN4" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="BN4" s="5" t="s">
+      <c r="BO4" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="BO4" s="5" t="s">
+      <c r="BP4" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="BP4" s="5" t="s">
+      <c r="BQ4" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="BQ4" s="5" t="s">
+      <c r="BR4" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="BR4" s="5" t="s">
+      <c r="BS4" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BS4" s="5" t="s">
+      <c r="BT4" s="5" t="s">
         <v>493</v>
       </c>
-      <c r="BT4" s="5" t="s">
+      <c r="BU4" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="BU4" s="5" t="s">
+      <c r="BV4" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="BV4" s="5" t="s">
+      <c r="BW4" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="BW4" s="5" t="s">
+      <c r="BX4" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="BX4" s="5" t="s">
+      <c r="BY4" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="BY4" s="5" t="s">
+      <c r="BZ4" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="BZ4" s="5" t="s">
+      <c r="CA4" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="CA4" s="5" t="s">
+      <c r="CB4" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="CB4" s="5" t="s">
+      <c r="CC4" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="CC4" s="5" t="s">
+      <c r="CD4" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="CD4" s="5" t="s">
+      <c r="CE4" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="CE4" s="5" t="s">
+      <c r="CF4" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="CF4" s="5" t="s">
+      <c r="CG4" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="CG4" s="5" t="s">
+      <c r="CH4" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="CH4" s="5" t="s">
+      <c r="CI4" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="CI4" s="5" t="s">
+      <c r="CJ4" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="CJ4" s="5" t="s">
+      <c r="CK4" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="CK4" s="5" t="s">
+      <c r="CL4" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="CL4" s="5" t="s">
+      <c r="CM4" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="CM4" s="5" t="s">
+      <c r="CN4" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="CN4" s="5" t="s">
+      <c r="CO4" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="CO4" s="5" t="s">
+      <c r="CP4" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="CP4" s="5" t="s">
+      <c r="CQ4" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="CQ4" s="5" t="s">
+      <c r="CR4" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="CR4" s="5" t="s">
+      <c r="CS4" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="CS4" s="5" t="s">
+      <c r="CT4" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="CT4" s="5" t="s">
+      <c r="CU4" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="CU4" s="5" t="s">
+      <c r="CV4" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="CV4" s="5" t="s">
+      <c r="CW4" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="CW4" s="5" t="s">
+      <c r="CX4" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="CX4" s="5" t="s">
+      <c r="CY4" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="CY4" s="5" t="s">
+      <c r="CZ4" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="CZ4" s="5" t="s">
+      <c r="DA4" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="DA4" s="5" t="s">
+      <c r="DB4" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="DB4" s="5" t="s">
+      <c r="DC4" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="DC4" s="5" t="s">
+      <c r="DD4" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="DD4" s="5" t="s">
+      <c r="DE4" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="DE4" s="5" t="s">
+      <c r="DF4" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="DF4" s="5" t="s">
+      <c r="DG4" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="DG4" s="5" t="s">
+      <c r="DH4" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="DH4" s="5" t="s">
+      <c r="DI4" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="DI4" s="5" t="s">
+      <c r="DJ4" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="DJ4" s="5" t="s">
+      <c r="DK4" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="DK4" s="5" t="s">
+      <c r="DL4" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="DL4" s="5" t="s">
+      <c r="DM4" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="DM4" s="5" t="s">
+      <c r="DN4" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="DN4" s="5" t="s">
+      <c r="DO4" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="DO4" s="5" t="s">
+      <c r="DP4" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="DP4" s="5" t="s">
+      <c r="DQ4" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="DQ4" s="5" t="s">
+      <c r="DR4" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="DR4" s="5" t="s">
+      <c r="DS4" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="DS4" s="5" t="s">
+      <c r="DT4" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="DT4" s="5" t="s">
+      <c r="DU4" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="DU4" s="5" t="s">
+      <c r="DV4" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="DV4" s="5" t="s">
+      <c r="DW4" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="DW4" s="5" t="s">
+      <c r="DX4" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="DX4" s="5" t="s">
+      <c r="DY4" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="DY4" s="5" t="s">
+      <c r="DZ4" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="DZ4" s="5" t="s">
+      <c r="EA4" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="EA4" s="5"/>
       <c r="EB4" s="5"/>
       <c r="EC4" s="5"/>
       <c r="ED4" s="5"/>
@@ -12141,8 +13602,9 @@
       <c r="FE4" s="5"/>
       <c r="FF4" s="5"/>
       <c r="FG4" s="5"/>
+      <c r="FH4" s="5"/>
     </row>
-    <row r="5" spans="1:163" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:164" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>46</v>
       </c>
@@ -12330,210 +13792,212 @@
         <v>5</v>
       </c>
       <c r="BK5" s="5">
+        <v>8.5</v>
+      </c>
+      <c r="BL5" s="5">
         <v>11.2</v>
       </c>
-      <c r="BL5" s="5">
+      <c r="BM5" s="5">
         <v>12.5</v>
       </c>
-      <c r="BM5" s="5">
+      <c r="BN5" s="5">
         <v>14</v>
       </c>
-      <c r="BN5" s="5">
+      <c r="BO5" s="5">
         <v>16</v>
       </c>
-      <c r="BO5" s="5">
+      <c r="BP5" s="5">
         <v>28</v>
       </c>
-      <c r="BP5" s="5">
+      <c r="BQ5" s="5">
         <v>33.5</v>
       </c>
-      <c r="BQ5" s="5">
+      <c r="BR5" s="5">
         <v>22.4</v>
       </c>
-      <c r="BR5" s="5">
+      <c r="BS5" s="5">
         <v>25</v>
       </c>
-      <c r="BS5" s="5">
+      <c r="BT5" s="5">
         <v>15.5</v>
       </c>
-      <c r="BT5" s="5">
+      <c r="BU5" s="5">
         <v>20</v>
       </c>
-      <c r="BU5" s="5">
+      <c r="BV5" s="5">
         <v>24</v>
       </c>
-      <c r="BV5" s="5">
+      <c r="BW5" s="5">
         <v>11.2</v>
       </c>
-      <c r="BW5" s="5">
+      <c r="BX5" s="5">
         <v>12.5</v>
       </c>
-      <c r="BX5" s="5">
+      <c r="BY5" s="5">
         <v>14</v>
       </c>
-      <c r="BY5" s="5">
+      <c r="BZ5" s="5">
         <v>22.4</v>
       </c>
-      <c r="BZ5" s="5">
+      <c r="CA5" s="5">
         <v>28</v>
       </c>
-      <c r="CA5" s="5">
+      <c r="CB5" s="5">
         <v>33.5</v>
       </c>
-      <c r="CB5" s="5">
+      <c r="CC5" s="5">
         <v>40</v>
       </c>
-      <c r="CC5" s="5">
+      <c r="CD5" s="5">
         <v>45</v>
       </c>
-      <c r="CD5" s="5">
+      <c r="CE5" s="5">
         <v>50</v>
       </c>
-      <c r="CE5" s="5">
+      <c r="CF5" s="5">
         <v>54</v>
       </c>
-      <c r="CF5" s="5">
+      <c r="CG5" s="5">
         <v>61.5</v>
       </c>
-      <c r="CG5" s="5">
+      <c r="CH5" s="5">
         <v>67</v>
       </c>
-      <c r="CH5" s="5">
+      <c r="CI5" s="5">
         <v>73.5</v>
       </c>
-      <c r="CI5" s="5">
+      <c r="CJ5" s="5">
         <v>78.5</v>
       </c>
-      <c r="CJ5" s="5">
+      <c r="CK5" s="5">
         <v>85</v>
       </c>
-      <c r="CK5" s="5">
+      <c r="CL5" s="5">
         <v>90</v>
       </c>
-      <c r="CL5" s="5">
+      <c r="CM5" s="5">
         <v>95</v>
       </c>
-      <c r="CM5" s="5">
+      <c r="CN5" s="5">
         <v>100</v>
       </c>
-      <c r="CN5" s="5">
+      <c r="CO5" s="5">
         <v>104</v>
       </c>
-      <c r="CO5" s="5">
+      <c r="CP5" s="5">
         <v>108</v>
       </c>
-      <c r="CP5" s="5">
+      <c r="CQ5" s="5">
         <v>117</v>
       </c>
-      <c r="CQ5" s="5">
+      <c r="CR5" s="5">
         <v>121</v>
       </c>
-      <c r="CR5" s="5">
+      <c r="CS5" s="5">
         <v>130</v>
       </c>
-      <c r="CS5" s="5">
+      <c r="CT5" s="5">
         <v>135</v>
       </c>
-      <c r="CT5" s="5">
+      <c r="CU5" s="5">
         <v>140</v>
       </c>
-      <c r="CU5" s="5">
+      <c r="CV5" s="5">
         <v>145</v>
       </c>
-      <c r="CV5" s="5">
+      <c r="CW5" s="5">
         <v>150</v>
       </c>
-      <c r="CW5" s="5">
+      <c r="CX5" s="5">
         <v>154</v>
       </c>
-      <c r="CX5" s="5">
+      <c r="CY5" s="5">
         <v>158</v>
       </c>
-      <c r="CY5" s="5">
+      <c r="CZ5" s="5">
         <v>162</v>
       </c>
-      <c r="CZ5" s="5">
+      <c r="DA5" s="5">
         <v>22.4</v>
       </c>
-      <c r="DA5" s="5">
+      <c r="DB5" s="5">
         <v>28</v>
       </c>
-      <c r="DB5" s="5">
+      <c r="DC5" s="5">
         <v>33.5</v>
       </c>
-      <c r="DC5" s="5">
+      <c r="DD5" s="5">
         <v>40</v>
       </c>
-      <c r="DD5" s="5">
+      <c r="DE5" s="5">
         <v>45</v>
       </c>
-      <c r="DE5" s="5">
+      <c r="DF5" s="5">
         <v>50</v>
       </c>
-      <c r="DF5" s="5">
+      <c r="DG5" s="5">
         <v>54</v>
       </c>
-      <c r="DG5" s="5">
+      <c r="DH5" s="5">
         <v>61.5</v>
       </c>
-      <c r="DH5" s="5">
+      <c r="DI5" s="5">
         <v>67</v>
       </c>
-      <c r="DI5" s="5">
+      <c r="DJ5" s="5">
         <v>73.5</v>
       </c>
-      <c r="DJ5" s="5">
+      <c r="DK5" s="5">
         <v>78.5</v>
       </c>
-      <c r="DK5" s="5">
+      <c r="DL5" s="5">
         <v>85</v>
       </c>
-      <c r="DL5" s="5">
+      <c r="DM5" s="5">
         <v>90</v>
       </c>
-      <c r="DM5" s="5">
+      <c r="DN5" s="5">
         <v>95</v>
       </c>
-      <c r="DN5" s="5">
+      <c r="DO5" s="5">
         <v>100</v>
       </c>
-      <c r="DO5" s="5">
+      <c r="DP5" s="5">
         <v>104</v>
       </c>
-      <c r="DP5" s="5">
+      <c r="DQ5" s="5">
         <v>108</v>
       </c>
-      <c r="DQ5" s="5">
+      <c r="DR5" s="5">
         <v>117</v>
       </c>
-      <c r="DR5" s="5">
+      <c r="DS5" s="5">
         <v>121</v>
       </c>
-      <c r="DS5" s="5">
+      <c r="DT5" s="5">
         <v>130</v>
       </c>
-      <c r="DT5" s="5">
+      <c r="DU5" s="5">
         <v>135</v>
       </c>
-      <c r="DU5" s="5">
+      <c r="DV5" s="5">
         <v>140</v>
       </c>
-      <c r="DV5" s="5">
+      <c r="DW5" s="5">
         <v>145</v>
       </c>
-      <c r="DW5" s="5">
+      <c r="DX5" s="5">
         <v>150</v>
       </c>
-      <c r="DX5" s="5">
+      <c r="DY5" s="5">
         <v>154</v>
       </c>
-      <c r="DY5" s="5">
+      <c r="DZ5" s="5">
         <v>158</v>
       </c>
-      <c r="DZ5" s="5">
+      <c r="EA5" s="5">
         <v>162</v>
       </c>
-      <c r="EA5" s="5"/>
       <c r="EB5" s="5"/>
       <c r="EC5" s="5"/>
       <c r="ED5" s="5"/>
@@ -12566,8 +14030,9 @@
       <c r="FE5" s="5"/>
       <c r="FF5" s="5"/>
       <c r="FG5" s="5"/>
+      <c r="FH5" s="5"/>
     </row>
-    <row r="6" spans="1:163" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:164" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>45</v>
       </c>
@@ -12754,211 +14219,213 @@
       <c r="BJ6" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="BK6" s="5">
+      <c r="BK6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="BL6" s="5">
         <v>100</v>
       </c>
-      <c r="BL6" s="5">
+      <c r="BM6" s="5">
         <v>112.5</v>
       </c>
-      <c r="BM6" s="5">
+      <c r="BN6" s="5">
         <v>125</v>
       </c>
-      <c r="BN6" s="5">
+      <c r="BO6" s="5">
         <v>150</v>
       </c>
-      <c r="BO6" s="5">
+      <c r="BP6" s="5">
         <v>250</v>
       </c>
-      <c r="BP6" s="5">
+      <c r="BQ6" s="5">
         <v>300</v>
       </c>
-      <c r="BQ6" s="5">
+      <c r="BR6" s="5">
         <v>200</v>
       </c>
-      <c r="BR6" s="5">
+      <c r="BS6" s="5">
         <v>223</v>
       </c>
-      <c r="BS6" s="5">
+      <c r="BT6" s="5">
         <v>140</v>
       </c>
-      <c r="BT6" s="5">
+      <c r="BU6" s="5">
         <v>180</v>
       </c>
-      <c r="BU6" s="5">
+      <c r="BV6" s="5">
         <v>215</v>
       </c>
-      <c r="BV6" s="5">
+      <c r="BW6" s="5">
         <v>100</v>
       </c>
-      <c r="BW6" s="5">
+      <c r="BX6" s="5">
         <v>112.5</v>
       </c>
-      <c r="BX6" s="5">
+      <c r="BY6" s="5">
         <v>125</v>
       </c>
-      <c r="BY6" s="5">
+      <c r="BZ6" s="5">
         <v>200</v>
       </c>
-      <c r="BZ6" s="5">
+      <c r="CA6" s="5">
         <v>250</v>
       </c>
-      <c r="CA6" s="5">
+      <c r="CB6" s="5">
         <v>300</v>
       </c>
-      <c r="CB6" s="5">
+      <c r="CC6" s="5">
         <v>350</v>
       </c>
-      <c r="CC6" s="5">
+      <c r="CD6" s="5">
         <v>400</v>
       </c>
-      <c r="CD6" s="5">
+      <c r="CE6" s="5">
         <v>450</v>
       </c>
-      <c r="CE6" s="5">
+      <c r="CF6" s="5">
         <v>500</v>
       </c>
-      <c r="CF6" s="5">
+      <c r="CG6" s="5">
         <v>550</v>
       </c>
-      <c r="CG6" s="5">
+      <c r="CH6" s="5">
         <v>600</v>
       </c>
-      <c r="CH6" s="5">
+      <c r="CI6" s="5">
         <v>650</v>
       </c>
-      <c r="CI6" s="5">
+      <c r="CJ6" s="5">
         <v>700</v>
       </c>
-      <c r="CJ6" s="5">
+      <c r="CK6" s="5">
         <v>750</v>
       </c>
-      <c r="CK6" s="5">
+      <c r="CL6" s="5">
         <v>800</v>
       </c>
-      <c r="CL6" s="5">
+      <c r="CM6" s="5">
         <v>850</v>
       </c>
-      <c r="CM6" s="5">
+      <c r="CN6" s="5">
         <v>900</v>
       </c>
-      <c r="CN6" s="5">
+      <c r="CO6" s="5">
         <v>950</v>
       </c>
-      <c r="CO6" s="5">
+      <c r="CP6" s="5">
         <v>1000</v>
       </c>
-      <c r="CP6" s="5">
+      <c r="CQ6" s="5">
         <v>1050</v>
       </c>
-      <c r="CQ6" s="5">
+      <c r="CR6" s="5">
         <v>1100</v>
       </c>
-      <c r="CR6" s="5">
+      <c r="CS6" s="5">
         <v>1150</v>
       </c>
-      <c r="CS6" s="5">
+      <c r="CT6" s="5">
         <v>1200</v>
       </c>
-      <c r="CT6" s="5">
+      <c r="CU6" s="5">
         <v>1250</v>
       </c>
-      <c r="CU6" s="5">
+      <c r="CV6" s="5">
         <v>1300</v>
       </c>
-      <c r="CV6" s="5">
+      <c r="CW6" s="5">
         <v>1350</v>
       </c>
-      <c r="CW6" s="5">
+      <c r="CX6" s="5">
         <v>1400</v>
       </c>
-      <c r="CX6" s="5">
+      <c r="CY6" s="5">
         <v>1450</v>
       </c>
-      <c r="CY6" s="5">
+      <c r="CZ6" s="5">
         <v>1500</v>
       </c>
-      <c r="CZ6" s="5">
+      <c r="DA6" s="5">
         <v>200</v>
       </c>
-      <c r="DA6" s="5">
+      <c r="DB6" s="5">
         <v>250</v>
       </c>
-      <c r="DB6" s="5">
+      <c r="DC6" s="5">
         <v>300</v>
       </c>
-      <c r="DC6" s="5">
+      <c r="DD6" s="5">
         <v>350</v>
       </c>
-      <c r="DD6" s="5">
+      <c r="DE6" s="5">
         <v>400</v>
       </c>
-      <c r="DE6" s="5">
+      <c r="DF6" s="5">
         <v>450</v>
       </c>
-      <c r="DF6" s="5">
+      <c r="DG6" s="5">
         <v>500</v>
       </c>
-      <c r="DG6" s="5">
+      <c r="DH6" s="5">
         <v>550</v>
       </c>
-      <c r="DH6" s="5">
+      <c r="DI6" s="5">
         <v>600</v>
       </c>
-      <c r="DI6" s="5">
+      <c r="DJ6" s="5">
         <v>650</v>
       </c>
-      <c r="DJ6" s="5">
+      <c r="DK6" s="5">
         <v>700</v>
       </c>
-      <c r="DK6" s="5">
+      <c r="DL6" s="5">
         <v>750</v>
       </c>
-      <c r="DL6" s="5">
+      <c r="DM6" s="5">
         <v>800</v>
       </c>
-      <c r="DM6" s="5">
+      <c r="DN6" s="5">
         <v>850</v>
       </c>
-      <c r="DN6" s="5">
+      <c r="DO6" s="5">
         <v>900</v>
       </c>
-      <c r="DO6" s="5">
+      <c r="DP6" s="5">
         <v>950</v>
       </c>
-      <c r="DP6" s="5">
+      <c r="DQ6" s="5">
         <v>1000</v>
       </c>
-      <c r="DQ6" s="5">
+      <c r="DR6" s="5">
         <v>1050</v>
       </c>
-      <c r="DR6" s="5">
+      <c r="DS6" s="5">
         <v>1100</v>
       </c>
-      <c r="DS6" s="5">
+      <c r="DT6" s="5">
         <v>1150</v>
       </c>
-      <c r="DT6" s="5">
+      <c r="DU6" s="5">
         <v>1200</v>
       </c>
-      <c r="DU6" s="5">
+      <c r="DV6" s="5">
         <v>1250</v>
       </c>
-      <c r="DV6" s="5">
+      <c r="DW6" s="5">
         <v>1300</v>
       </c>
-      <c r="DW6" s="5">
+      <c r="DX6" s="5">
         <v>1350</v>
       </c>
-      <c r="DX6" s="5">
+      <c r="DY6" s="5">
         <v>1400</v>
       </c>
-      <c r="DY6" s="5">
+      <c r="DZ6" s="5">
         <v>1450</v>
       </c>
-      <c r="DZ6" s="5">
+      <c r="EA6" s="5">
         <v>1500</v>
       </c>
-      <c r="EA6" s="5"/>
       <c r="EB6" s="5"/>
       <c r="EC6" s="5"/>
       <c r="ED6" s="5"/>
@@ -12991,8 +14458,9 @@
       <c r="FE6" s="5"/>
       <c r="FF6" s="5"/>
       <c r="FG6" s="5"/>
+      <c r="FH6" s="5"/>
     </row>
-    <row r="7" spans="1:163" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:164" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>48</v>
       </c>
@@ -13180,7 +14648,7 @@
         <v>9</v>
       </c>
       <c r="BK7" s="5" t="s">
-        <v>127</v>
+        <v>9</v>
       </c>
       <c r="BL7" s="5" t="s">
         <v>127</v>
@@ -13192,28 +14660,28 @@
         <v>127</v>
       </c>
       <c r="BO7" s="5" t="s">
-        <v>494</v>
+        <v>127</v>
       </c>
       <c r="BP7" s="5" t="s">
         <v>494</v>
       </c>
       <c r="BQ7" s="5" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="BR7" s="5" t="s">
         <v>495</v>
       </c>
       <c r="BS7" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="BT7" s="5" t="s">
         <v>127</v>
-      </c>
-      <c r="BT7" s="5" t="s">
-        <v>494</v>
       </c>
       <c r="BU7" s="5" t="s">
         <v>494</v>
       </c>
       <c r="BV7" s="5" t="s">
-        <v>127</v>
+        <v>494</v>
       </c>
       <c r="BW7" s="5" t="s">
         <v>127</v>
@@ -13222,7 +14690,7 @@
         <v>127</v>
       </c>
       <c r="BY7" s="5" t="s">
-        <v>494</v>
+        <v>127</v>
       </c>
       <c r="BZ7" s="5" t="s">
         <v>494</v>
@@ -13383,7 +14851,9 @@
       <c r="DZ7" s="5" t="s">
         <v>494</v>
       </c>
-      <c r="EA7" s="5"/>
+      <c r="EA7" s="5" t="s">
+        <v>494</v>
+      </c>
       <c r="EB7" s="5"/>
       <c r="EC7" s="5"/>
       <c r="ED7" s="5"/>
@@ -13416,8 +14886,9 @@
       <c r="FE7" s="5"/>
       <c r="FF7" s="5"/>
       <c r="FG7" s="5"/>
+      <c r="FH7" s="5"/>
     </row>
-    <row r="8" spans="1:163" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:164" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>47</v>
       </c>
@@ -13605,210 +15076,212 @@
         <v>1.52</v>
       </c>
       <c r="BK8" s="5">
+        <v>2.67</v>
+      </c>
+      <c r="BL8" s="5">
         <v>2.25</v>
       </c>
-      <c r="BL8" s="5">
+      <c r="BM8" s="5">
         <v>2.66</v>
       </c>
-      <c r="BM8" s="5">
+      <c r="BN8" s="5">
         <v>3.08</v>
       </c>
-      <c r="BN8" s="5">
+      <c r="BO8" s="5">
         <v>3.97</v>
       </c>
-      <c r="BO8" s="5">
+      <c r="BP8" s="5">
         <v>6.72</v>
       </c>
-      <c r="BP8" s="5">
+      <c r="BQ8" s="5">
         <v>8.93</v>
       </c>
-      <c r="BQ8" s="5">
+      <c r="BR8" s="5">
         <v>6.3</v>
       </c>
-      <c r="BR8" s="5">
+      <c r="BS8" s="5">
         <v>7.8</v>
       </c>
-      <c r="BS8" s="5">
+      <c r="BT8" s="5">
         <v>4.3899999999999997</v>
       </c>
-      <c r="BT8" s="5">
+      <c r="BU8" s="5">
         <v>5.91</v>
       </c>
-      <c r="BU8" s="5">
+      <c r="BV8" s="5">
         <v>7.51</v>
       </c>
-      <c r="BV8" s="5">
+      <c r="BW8" s="5">
         <v>2.81</v>
       </c>
-      <c r="BW8" s="5">
+      <c r="BX8" s="5">
         <v>3.28</v>
       </c>
-      <c r="BX8" s="5">
+      <c r="BY8" s="5">
         <v>4.01</v>
       </c>
-      <c r="BY8" s="5">
+      <c r="BZ8" s="5">
         <v>5.32</v>
       </c>
-      <c r="BZ8" s="5">
+      <c r="CA8" s="5">
         <v>7.26</v>
       </c>
-      <c r="CA8" s="5">
+      <c r="CB8" s="5">
         <v>9.26</v>
       </c>
-      <c r="CB8" s="5">
+      <c r="CC8" s="5">
         <v>11.35</v>
       </c>
-      <c r="CC8" s="5">
+      <c r="CD8" s="5">
         <v>12.15</v>
       </c>
-      <c r="CD8" s="5">
+      <c r="CE8" s="5">
         <v>14.82</v>
       </c>
-      <c r="CE8" s="5">
+      <c r="CF8" s="5">
         <v>16.239999999999998</v>
       </c>
-      <c r="CF8" s="5">
+      <c r="CG8" s="5">
         <v>16.52</v>
       </c>
-      <c r="CG8" s="5">
+      <c r="CH8" s="5">
         <v>18.52</v>
       </c>
-      <c r="CH8" s="5">
+      <c r="CI8" s="5">
         <v>20.61</v>
       </c>
-      <c r="CI8" s="5">
+      <c r="CJ8" s="5">
         <v>21.41</v>
       </c>
-      <c r="CJ8" s="5">
+      <c r="CK8" s="5">
         <v>23.5</v>
       </c>
-      <c r="CK8" s="5">
+      <c r="CL8" s="5">
         <v>26.17</v>
       </c>
-      <c r="CL8" s="5">
+      <c r="CM8" s="5">
         <v>26.97</v>
       </c>
-      <c r="CM8" s="5">
+      <c r="CN8" s="5">
         <v>29.64</v>
       </c>
-      <c r="CN8" s="5">
+      <c r="CO8" s="5">
         <v>31.06</v>
       </c>
-      <c r="CO8" s="5">
+      <c r="CP8" s="5">
         <v>32.479999999999997</v>
       </c>
-      <c r="CP8" s="5">
+      <c r="CQ8" s="5">
         <v>33.340000000000003</v>
       </c>
-      <c r="CQ8" s="5">
+      <c r="CR8" s="5">
         <v>34.76</v>
       </c>
-      <c r="CR8" s="5">
+      <c r="CS8" s="5">
         <v>37.520000000000003</v>
       </c>
-      <c r="CS8" s="5">
+      <c r="CT8" s="5">
         <v>38.32</v>
       </c>
-      <c r="CT8" s="5">
+      <c r="CU8" s="5">
         <v>40.99</v>
       </c>
-      <c r="CU8" s="5">
+      <c r="CV8" s="5">
         <v>41.79</v>
       </c>
-      <c r="CV8" s="5">
+      <c r="CW8" s="5">
         <v>44.46</v>
       </c>
-      <c r="CW8" s="5">
+      <c r="CX8" s="5">
         <v>45.88</v>
       </c>
-      <c r="CX8" s="5">
+      <c r="CY8" s="5">
         <v>47.3</v>
       </c>
-      <c r="CY8" s="5">
+      <c r="CZ8" s="5">
         <v>48.72</v>
       </c>
-      <c r="CZ8" s="5">
+      <c r="DA8" s="5">
         <v>5.65</v>
       </c>
-      <c r="DA8" s="5">
+      <c r="DB8" s="5">
         <v>7.09</v>
       </c>
-      <c r="DB8" s="5">
+      <c r="DC8" s="5">
         <v>9.9700000000000006</v>
       </c>
-      <c r="DC8" s="5">
+      <c r="DD8" s="5">
         <v>12.08</v>
       </c>
-      <c r="DD8" s="5">
+      <c r="DE8" s="5">
         <v>13.92</v>
       </c>
-      <c r="DE8" s="5">
+      <c r="DF8" s="5">
         <v>15.07</v>
       </c>
-      <c r="DF8" s="5">
+      <c r="DG8" s="5">
         <v>16.5</v>
       </c>
-      <c r="DG8" s="5">
+      <c r="DH8" s="5">
         <v>17.059999999999999</v>
       </c>
-      <c r="DH8" s="5">
+      <c r="DI8" s="5">
         <v>19.940000000000001</v>
       </c>
-      <c r="DI8" s="5">
+      <c r="DJ8" s="5">
         <v>22.05</v>
       </c>
-      <c r="DJ8" s="5">
+      <c r="DK8" s="5">
         <v>23.89</v>
       </c>
-      <c r="DK8" s="5">
+      <c r="DL8" s="5">
         <v>26</v>
       </c>
-      <c r="DL8" s="5">
+      <c r="DM8" s="5">
         <v>27.15</v>
       </c>
-      <c r="DM8" s="5">
+      <c r="DN8" s="5">
         <v>28.99</v>
       </c>
-      <c r="DN8" s="5">
+      <c r="DO8" s="5">
         <v>30.14</v>
       </c>
-      <c r="DO8" s="5">
+      <c r="DP8" s="5">
         <v>31.57</v>
       </c>
-      <c r="DP8" s="5">
+      <c r="DQ8" s="5">
         <v>33</v>
       </c>
-      <c r="DQ8" s="5">
+      <c r="DR8" s="5">
         <v>35.01</v>
       </c>
-      <c r="DR8" s="5">
+      <c r="DS8" s="5">
         <v>36.44</v>
       </c>
-      <c r="DS8" s="5">
+      <c r="DT8" s="5">
         <v>39.229999999999997</v>
       </c>
-      <c r="DT8" s="5">
+      <c r="DU8" s="5">
         <v>41.07</v>
       </c>
-      <c r="DU8" s="5">
+      <c r="DV8" s="5">
         <v>42.22</v>
       </c>
-      <c r="DV8" s="5">
+      <c r="DW8" s="5">
         <v>44.06</v>
       </c>
-      <c r="DW8" s="5">
+      <c r="DX8" s="5">
         <v>45.21</v>
       </c>
-      <c r="DX8" s="5">
+      <c r="DY8" s="5">
         <v>46.64</v>
       </c>
-      <c r="DY8" s="5">
+      <c r="DZ8" s="5">
         <v>48.07</v>
       </c>
-      <c r="DZ8" s="5">
+      <c r="EA8" s="5">
         <v>49.5</v>
       </c>
-      <c r="EA8" s="5"/>
       <c r="EB8" s="5"/>
       <c r="EC8" s="5"/>
       <c r="ED8" s="5"/>
@@ -13841,8 +15314,9 @@
       <c r="FE8" s="5"/>
       <c r="FF8" s="5"/>
       <c r="FG8" s="5"/>
+      <c r="FH8" s="5"/>
     </row>
-    <row r="9" spans="1:163" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:164" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>50</v>
       </c>
@@ -14030,10 +15504,10 @@
         <v>9.6999999999999993</v>
       </c>
       <c r="BK9" s="5">
+        <v>16</v>
+      </c>
+      <c r="BL9" s="5">
         <v>20</v>
-      </c>
-      <c r="BL9" s="5">
-        <v>27</v>
       </c>
       <c r="BM9" s="5">
         <v>27</v>
@@ -14042,198 +15516,200 @@
         <v>27</v>
       </c>
       <c r="BO9" s="5">
+        <v>27</v>
+      </c>
+      <c r="BP9" s="5">
         <v>22</v>
       </c>
-      <c r="BP9" s="5">
+      <c r="BQ9" s="5">
         <v>24</v>
-      </c>
-      <c r="BQ9" s="5">
-        <v>26.5</v>
       </c>
       <c r="BR9" s="5">
         <v>26.5</v>
       </c>
       <c r="BS9" s="5">
+        <v>26.5</v>
+      </c>
+      <c r="BT9" s="5">
         <v>21.1</v>
-      </c>
-      <c r="BT9" s="5">
-        <v>18.5</v>
       </c>
       <c r="BU9" s="5">
         <v>18.5</v>
       </c>
       <c r="BV9" s="5">
+        <v>18.5</v>
+      </c>
+      <c r="BW9" s="5">
         <v>17.5</v>
-      </c>
-      <c r="BW9" s="5">
-        <v>27</v>
       </c>
       <c r="BX9" s="5">
         <v>27</v>
       </c>
       <c r="BY9" s="5">
+        <v>27</v>
+      </c>
+      <c r="BZ9" s="5">
         <v>16.100000000000001</v>
       </c>
-      <c r="BZ9" s="5">
+      <c r="CA9" s="5">
         <v>21.2</v>
       </c>
-      <c r="CA9" s="5">
+      <c r="CB9" s="5">
         <v>22.5</v>
       </c>
-      <c r="CB9" s="5">
+      <c r="CC9" s="5">
         <v>30.2</v>
       </c>
-      <c r="CC9" s="5">
+      <c r="CD9" s="5">
         <v>33.700000000000003</v>
       </c>
-      <c r="CD9" s="5">
+      <c r="CE9" s="5">
         <v>34.5</v>
       </c>
-      <c r="CE9" s="5">
+      <c r="CF9" s="5">
         <v>38.5</v>
       </c>
-      <c r="CF9" s="5">
+      <c r="CG9" s="5">
         <v>43.7</v>
       </c>
-      <c r="CG9" s="5">
+      <c r="CH9" s="5">
         <v>45</v>
       </c>
-      <c r="CH9" s="5">
+      <c r="CI9" s="5">
         <v>52.7</v>
       </c>
-      <c r="CI9" s="5">
+      <c r="CJ9" s="5">
         <v>56.2</v>
       </c>
-      <c r="CJ9" s="5">
+      <c r="CK9" s="5">
         <v>63.9</v>
       </c>
-      <c r="CK9" s="5">
+      <c r="CL9" s="5">
         <v>64.7</v>
       </c>
-      <c r="CL9" s="5">
+      <c r="CM9" s="5">
         <v>68.2</v>
       </c>
-      <c r="CM9" s="5">
+      <c r="CN9" s="5">
         <v>69</v>
       </c>
-      <c r="CN9" s="5">
+      <c r="CO9" s="5">
         <v>73</v>
       </c>
-      <c r="CO9" s="5">
+      <c r="CP9" s="5">
         <v>77</v>
       </c>
-      <c r="CP9" s="5">
+      <c r="CQ9" s="5">
         <v>79.5</v>
       </c>
-      <c r="CQ9" s="5">
+      <c r="CR9" s="5">
         <v>83.5</v>
       </c>
-      <c r="CR9" s="5">
+      <c r="CS9" s="5">
         <v>94.9</v>
       </c>
-      <c r="CS9" s="5">
+      <c r="CT9" s="5">
         <v>98.4</v>
       </c>
-      <c r="CT9" s="5">
+      <c r="CU9" s="5">
         <v>99.2</v>
       </c>
-      <c r="CU9" s="5">
+      <c r="CV9" s="5">
         <v>102.7</v>
       </c>
-      <c r="CV9" s="5">
+      <c r="CW9" s="5">
         <v>103.5</v>
       </c>
-      <c r="CW9" s="5">
+      <c r="CX9" s="5">
         <v>107.5</v>
       </c>
-      <c r="CX9" s="5">
+      <c r="CY9" s="5">
         <v>111.5</v>
       </c>
-      <c r="CY9" s="5">
+      <c r="CZ9" s="5">
         <v>115.5</v>
       </c>
-      <c r="CZ9" s="5">
+      <c r="DA9" s="5">
         <v>16.100000000000001</v>
       </c>
-      <c r="DA9" s="5">
+      <c r="DB9" s="5">
         <v>21.5</v>
       </c>
-      <c r="DB9" s="5">
+      <c r="DC9" s="5">
         <v>22.9</v>
       </c>
-      <c r="DC9" s="5">
+      <c r="DD9" s="5">
         <v>30.2</v>
       </c>
-      <c r="DD9" s="5">
+      <c r="DE9" s="5">
         <v>34</v>
       </c>
-      <c r="DE9" s="5">
+      <c r="DF9" s="5">
         <v>34.700000000000003</v>
       </c>
-      <c r="DF9" s="5">
+      <c r="DG9" s="5">
         <v>39.700000000000003</v>
       </c>
-      <c r="DG9" s="5">
+      <c r="DH9" s="5">
         <v>44.4</v>
       </c>
-      <c r="DH9" s="5">
+      <c r="DI9" s="5">
         <v>45.8</v>
       </c>
-      <c r="DI9" s="5">
+      <c r="DJ9" s="5">
         <v>53.1</v>
       </c>
-      <c r="DJ9" s="5">
+      <c r="DK9" s="5">
         <v>56.9</v>
       </c>
-      <c r="DK9" s="5">
+      <c r="DL9" s="5">
         <v>64.2</v>
       </c>
-      <c r="DL9" s="5">
+      <c r="DM9" s="5">
         <v>64.900000000000006</v>
       </c>
-      <c r="DM9" s="5">
+      <c r="DN9" s="5">
         <v>68.7</v>
       </c>
-      <c r="DN9" s="5">
+      <c r="DO9" s="5">
         <v>69.400000000000006</v>
       </c>
-      <c r="DO9" s="5">
+      <c r="DP9" s="5">
         <v>74.400000000000006</v>
       </c>
-      <c r="DP9" s="5">
+      <c r="DQ9" s="5">
         <v>79.400000000000006</v>
       </c>
-      <c r="DQ9" s="5">
+      <c r="DR9" s="5">
         <v>80.5</v>
       </c>
-      <c r="DR9" s="5">
+      <c r="DS9" s="5">
         <v>85.5</v>
       </c>
-      <c r="DS9" s="5">
+      <c r="DT9" s="5">
         <v>95.1</v>
       </c>
-      <c r="DT9" s="5">
+      <c r="DU9" s="5">
         <v>98.9</v>
       </c>
-      <c r="DU9" s="5">
+      <c r="DV9" s="5">
         <v>99.6</v>
       </c>
-      <c r="DV9" s="5">
+      <c r="DW9" s="5">
         <v>103.4</v>
       </c>
-      <c r="DW9" s="5">
+      <c r="DX9" s="5">
         <v>104.1</v>
       </c>
-      <c r="DX9" s="5">
+      <c r="DY9" s="5">
         <v>109.1</v>
       </c>
-      <c r="DY9" s="5">
+      <c r="DZ9" s="5">
         <v>114.1</v>
       </c>
-      <c r="DZ9" s="5">
+      <c r="EA9" s="5">
         <v>119.1</v>
       </c>
-      <c r="EA9" s="5"/>
       <c r="EB9" s="5"/>
       <c r="EC9" s="5"/>
       <c r="ED9" s="5"/>
@@ -14266,8 +15742,9 @@
       <c r="FE9" s="5"/>
       <c r="FF9" s="5"/>
       <c r="FG9" s="5"/>
+      <c r="FH9" s="5"/>
     </row>
-    <row r="10" spans="1:163" ht="25.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:164" ht="25.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>49</v>
       </c>
@@ -14451,10 +15928,10 @@
         <v>10</v>
       </c>
       <c r="BK10" s="5">
+        <v>20</v>
+      </c>
+      <c r="BL10" s="5">
         <v>25</v>
-      </c>
-      <c r="BL10" s="5">
-        <v>30</v>
       </c>
       <c r="BM10" s="5">
         <v>30</v>
@@ -14463,10 +15940,10 @@
         <v>30</v>
       </c>
       <c r="BO10" s="5">
+        <v>30</v>
+      </c>
+      <c r="BP10" s="5">
         <v>25</v>
-      </c>
-      <c r="BP10" s="5">
-        <v>30</v>
       </c>
       <c r="BQ10" s="5">
         <v>30</v>
@@ -14478,7 +15955,7 @@
         <v>30</v>
       </c>
       <c r="BT10" s="5">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="BU10" s="5">
         <v>25</v>
@@ -14487,46 +15964,46 @@
         <v>25</v>
       </c>
       <c r="BW10" s="5">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="BX10" s="5">
         <v>30</v>
       </c>
       <c r="BY10" s="5">
+        <v>30</v>
+      </c>
+      <c r="BZ10" s="5">
         <v>20</v>
-      </c>
-      <c r="BZ10" s="5">
-        <v>25</v>
       </c>
       <c r="CA10" s="5">
         <v>25</v>
       </c>
       <c r="CB10" s="5">
+        <v>25</v>
+      </c>
+      <c r="CC10" s="5">
         <v>35</v>
-      </c>
-      <c r="CC10" s="5">
-        <v>40</v>
       </c>
       <c r="CD10" s="5">
         <v>40</v>
       </c>
       <c r="CE10" s="5">
+        <v>40</v>
+      </c>
+      <c r="CF10" s="5">
         <v>45</v>
-      </c>
-      <c r="CF10" s="5">
-        <v>50</v>
       </c>
       <c r="CG10" s="5">
         <v>50</v>
       </c>
       <c r="CH10" s="5">
+        <v>50</v>
+      </c>
+      <c r="CI10" s="5">
         <v>60</v>
       </c>
-      <c r="CI10" s="5">
+      <c r="CJ10" s="5">
         <v>70</v>
-      </c>
-      <c r="CJ10" s="5">
-        <v>80</v>
       </c>
       <c r="CK10" s="5">
         <v>80</v>
@@ -14538,7 +16015,7 @@
         <v>80</v>
       </c>
       <c r="CN10" s="5">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="CO10" s="5">
         <v>90</v>
@@ -14547,10 +16024,10 @@
         <v>90</v>
       </c>
       <c r="CQ10" s="5">
+        <v>90</v>
+      </c>
+      <c r="CR10" s="5">
         <v>100</v>
-      </c>
-      <c r="CR10" s="5">
-        <v>110</v>
       </c>
       <c r="CS10" s="5">
         <v>110</v>
@@ -14559,7 +16036,7 @@
         <v>110</v>
       </c>
       <c r="CU10" s="5">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="CV10" s="5">
         <v>125</v>
@@ -14571,43 +16048,43 @@
         <v>125</v>
       </c>
       <c r="CY10" s="5">
+        <v>125</v>
+      </c>
+      <c r="CZ10" s="5">
         <v>150</v>
       </c>
-      <c r="CZ10" s="5">
+      <c r="DA10" s="5">
         <v>20</v>
       </c>
-      <c r="DA10" s="5">
+      <c r="DB10" s="5">
         <v>25</v>
       </c>
-      <c r="DB10" s="5">
+      <c r="DC10" s="5">
         <v>30</v>
       </c>
-      <c r="DC10" s="5">
+      <c r="DD10" s="5">
         <v>35</v>
-      </c>
-      <c r="DD10" s="5">
-        <v>40</v>
       </c>
       <c r="DE10" s="5">
         <v>40</v>
       </c>
       <c r="DF10" s="5">
+        <v>40</v>
+      </c>
+      <c r="DG10" s="5">
         <v>45</v>
       </c>
-      <c r="DG10" s="5">
+      <c r="DH10" s="5">
         <v>50</v>
-      </c>
-      <c r="DH10" s="5">
-        <v>60</v>
       </c>
       <c r="DI10" s="5">
         <v>60</v>
       </c>
       <c r="DJ10" s="5">
+        <v>60</v>
+      </c>
+      <c r="DK10" s="5">
         <v>70</v>
-      </c>
-      <c r="DK10" s="5">
-        <v>80</v>
       </c>
       <c r="DL10" s="5">
         <v>80</v>
@@ -14619,7 +16096,7 @@
         <v>80</v>
       </c>
       <c r="DO10" s="5">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="DP10" s="5">
         <v>90</v>
@@ -14628,10 +16105,10 @@
         <v>90</v>
       </c>
       <c r="DR10" s="5">
+        <v>90</v>
+      </c>
+      <c r="DS10" s="5">
         <v>100</v>
-      </c>
-      <c r="DS10" s="5">
-        <v>110</v>
       </c>
       <c r="DT10" s="5">
         <v>110</v>
@@ -14640,7 +16117,7 @@
         <v>110</v>
       </c>
       <c r="DV10" s="5">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="DW10" s="5">
         <v>125</v>
@@ -14649,12 +16126,14 @@
         <v>125</v>
       </c>
       <c r="DY10" s="5">
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="DZ10" s="5">
         <v>150</v>
       </c>
-      <c r="EA10" s="5"/>
+      <c r="EA10" s="5">
+        <v>150</v>
+      </c>
       <c r="EB10" s="5"/>
       <c r="EC10" s="5"/>
       <c r="ED10" s="5"/>
@@ -14687,8 +16166,9 @@
       <c r="FE10" s="5"/>
       <c r="FF10" s="5"/>
       <c r="FG10" s="5"/>
+      <c r="FH10" s="5"/>
     </row>
-    <row r="11" spans="1:163" ht="25.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:164" ht="25.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
         <v>58</v>
       </c>
@@ -14873,8 +16353,8 @@
       <c r="BJ11" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="BK11" s="15">
-        <v>40</v>
+      <c r="BK11" s="15" t="s">
+        <v>37</v>
       </c>
       <c r="BL11" s="15">
         <v>40</v>
@@ -14885,8 +16365,8 @@
       <c r="BN11" s="15">
         <v>40</v>
       </c>
-      <c r="BO11" s="15" t="s">
-        <v>37</v>
+      <c r="BO11" s="15">
+        <v>40</v>
       </c>
       <c r="BP11" s="15" t="s">
         <v>37</v>
@@ -14915,8 +16395,8 @@
       <c r="BX11" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="BY11" s="15">
-        <v>78.400000000000006</v>
+      <c r="BY11" s="15" t="s">
+        <v>37</v>
       </c>
       <c r="BZ11" s="15">
         <v>78.400000000000006</v>
@@ -15077,7 +16557,9 @@
       <c r="DZ11" s="15">
         <v>78.400000000000006</v>
       </c>
-      <c r="EA11" s="15"/>
+      <c r="EA11" s="15">
+        <v>78.400000000000006</v>
+      </c>
       <c r="EB11" s="15"/>
       <c r="EC11" s="15"/>
       <c r="ED11" s="15"/>
@@ -15110,8 +16592,9 @@
       <c r="FE11" s="15"/>
       <c r="FF11" s="15"/>
       <c r="FG11" s="15"/>
+      <c r="FH11" s="15"/>
     </row>
-    <row r="12" spans="1:163" ht="60" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:164" ht="60" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
         <v>51</v>
       </c>
@@ -15299,7 +16782,7 @@
         <v>40</v>
       </c>
       <c r="BK12" s="15" t="s">
-        <v>125</v>
+        <v>570</v>
       </c>
       <c r="BL12" s="15" t="s">
         <v>125</v>
@@ -15311,13 +16794,13 @@
         <v>125</v>
       </c>
       <c r="BO12" s="15" t="s">
-        <v>143</v>
+        <v>125</v>
       </c>
       <c r="BP12" s="15" t="s">
         <v>143</v>
       </c>
       <c r="BQ12" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="BR12" s="15" t="s">
         <v>144</v>
@@ -15332,7 +16815,7 @@
         <v>144</v>
       </c>
       <c r="BV12" s="15" t="s">
-        <v>74</v>
+        <v>144</v>
       </c>
       <c r="BW12" s="15" t="s">
         <v>74</v>
@@ -15341,7 +16824,7 @@
         <v>74</v>
       </c>
       <c r="BY12" s="15" t="s">
-        <v>177</v>
+        <v>74</v>
       </c>
       <c r="BZ12" s="15" t="s">
         <v>177</v>
@@ -15350,7 +16833,7 @@
         <v>177</v>
       </c>
       <c r="CB12" s="15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="CC12" s="15" t="s">
         <v>178</v>
@@ -15362,43 +16845,43 @@
         <v>178</v>
       </c>
       <c r="CF12" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="CG12" s="15" t="s">
         <v>179</v>
       </c>
       <c r="CH12" s="15" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="CI12" s="15" t="s">
         <v>180</v>
       </c>
       <c r="CJ12" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="CK12" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="CK12" s="15" t="s">
+      <c r="CL12" s="15" t="s">
         <v>182</v>
       </c>
-      <c r="CL12" s="15" t="s">
+      <c r="CM12" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="CM12" s="15" t="s">
+      <c r="CN12" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="CN12" s="15" t="s">
+      <c r="CO12" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="CO12" s="15" t="s">
+      <c r="CP12" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="CP12" s="15" t="s">
+      <c r="CQ12" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="CQ12" s="15" t="s">
+      <c r="CR12" s="15" t="s">
         <v>188</v>
-      </c>
-      <c r="CR12" s="15" t="s">
-        <v>189</v>
       </c>
       <c r="CS12" s="15" t="s">
         <v>189</v>
@@ -15422,7 +16905,7 @@
         <v>189</v>
       </c>
       <c r="CZ12" s="15" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="DA12" s="15" t="s">
         <v>177</v>
@@ -15431,7 +16914,7 @@
         <v>177</v>
       </c>
       <c r="DC12" s="15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="DD12" s="15" t="s">
         <v>178</v>
@@ -15443,43 +16926,43 @@
         <v>178</v>
       </c>
       <c r="DG12" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="DH12" s="15" t="s">
         <v>179</v>
       </c>
       <c r="DI12" s="15" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="DJ12" s="15" t="s">
         <v>180</v>
       </c>
       <c r="DK12" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="DL12" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="DL12" s="15" t="s">
+      <c r="DM12" s="15" t="s">
         <v>182</v>
       </c>
-      <c r="DM12" s="15" t="s">
+      <c r="DN12" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="DN12" s="15" t="s">
+      <c r="DO12" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="DO12" s="15" t="s">
+      <c r="DP12" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="DP12" s="15" t="s">
+      <c r="DQ12" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="DQ12" s="15" t="s">
+      <c r="DR12" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="DR12" s="15" t="s">
+      <c r="DS12" s="15" t="s">
         <v>188</v>
-      </c>
-      <c r="DS12" s="15" t="s">
-        <v>189</v>
       </c>
       <c r="DT12" s="15" t="s">
         <v>189</v>
@@ -15502,7 +16985,9 @@
       <c r="DZ12" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="EA12" s="15"/>
+      <c r="EA12" s="15" t="s">
+        <v>189</v>
+      </c>
       <c r="EB12" s="15"/>
       <c r="EC12" s="15"/>
       <c r="ED12" s="15"/>
@@ -15533,8 +17018,9 @@
       <c r="FC12" s="15"/>
       <c r="FD12" s="15"/>
       <c r="FE12" s="15"/>
+      <c r="FF12" s="15"/>
     </row>
-    <row r="13" spans="1:163" ht="25.35" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:164" ht="25.35" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="17" t="s">
         <v>54</v>
       </c>
@@ -15732,7 +17218,7 @@
         <v>56</v>
       </c>
       <c r="BO13" s="12" t="s">
-        <v>145</v>
+        <v>56</v>
       </c>
       <c r="BP13" s="12" t="s">
         <v>145</v>
@@ -15753,7 +17239,7 @@
         <v>145</v>
       </c>
       <c r="BV13" s="12" t="s">
-        <v>56</v>
+        <v>145</v>
       </c>
       <c r="BW13" s="12" t="s">
         <v>56</v>
@@ -15762,7 +17248,7 @@
         <v>56</v>
       </c>
       <c r="BY13" s="12" t="s">
-        <v>538</v>
+        <v>56</v>
       </c>
       <c r="BZ13" s="12" t="s">
         <v>538</v>
@@ -15843,7 +17329,7 @@
         <v>538</v>
       </c>
       <c r="CZ13" s="12" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="DA13" s="12" t="s">
         <v>539</v>
@@ -15923,7 +17409,9 @@
       <c r="DZ13" s="12" t="s">
         <v>539</v>
       </c>
-      <c r="EA13" s="12"/>
+      <c r="EA13" s="12" t="s">
+        <v>539</v>
+      </c>
       <c r="EB13" s="12"/>
       <c r="EC13" s="12"/>
       <c r="ED13" s="12"/>
@@ -15956,8 +17444,9 @@
       <c r="FE13" s="12"/>
       <c r="FF13" s="12"/>
       <c r="FG13" s="12"/>
+      <c r="FH13" s="12"/>
     </row>
-    <row r="14" spans="1:163" ht="25.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:164" ht="25.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="17" t="s">
         <v>542</v>
       </c>
@@ -16140,7 +17629,9 @@
       <c r="BJ14" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="BK14" s="21"/>
+      <c r="BK14" s="28" t="s">
+        <v>37</v>
+      </c>
       <c r="BL14" s="21"/>
       <c r="BM14" s="21"/>
       <c r="BN14" s="21"/>
@@ -16241,8 +17732,9 @@
       <c r="FE14" s="21"/>
       <c r="FF14" s="21"/>
       <c r="FG14" s="21"/>
+      <c r="FH14" s="21"/>
     </row>
-    <row r="15" spans="1:163" s="56" customFormat="1" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:164" s="56" customFormat="1" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="52" t="s">
         <v>562</v>
       </c>
@@ -16255,7 +17747,318 @@
       <c r="D15" s="54" t="s">
         <v>564</v>
       </c>
-      <c r="E15" s="55"/>
+      <c r="E15" s="55">
+        <v>20600</v>
+      </c>
+      <c r="F15" s="56">
+        <v>23800</v>
+      </c>
+      <c r="G15" s="56">
+        <v>25100</v>
+      </c>
+      <c r="H15" s="56">
+        <v>30000</v>
+      </c>
+      <c r="I15" s="56">
+        <v>34260</v>
+      </c>
+      <c r="J15" s="56">
+        <v>39960</v>
+      </c>
+      <c r="K15" s="56">
+        <v>44460</v>
+      </c>
+      <c r="L15" s="56">
+        <v>51660</v>
+      </c>
+      <c r="M15" s="56">
+        <v>56660</v>
+      </c>
+      <c r="N15" s="56">
+        <v>26500</v>
+      </c>
+      <c r="O15" s="56">
+        <v>29700</v>
+      </c>
+      <c r="P15" s="56">
+        <v>32700</v>
+      </c>
+      <c r="Q15" s="56">
+        <v>35400</v>
+      </c>
+      <c r="R15" s="56">
+        <v>39460</v>
+      </c>
+      <c r="S15" s="56">
+        <v>44960</v>
+      </c>
+      <c r="T15" s="56">
+        <v>47660</v>
+      </c>
+      <c r="AD15" s="56">
+        <v>19700</v>
+      </c>
+      <c r="AE15" s="56">
+        <v>22600</v>
+      </c>
+      <c r="AF15" s="56">
+        <v>24300</v>
+      </c>
+      <c r="AG15" s="56">
+        <v>27800</v>
+      </c>
+      <c r="AH15" s="56">
+        <v>33360</v>
+      </c>
+      <c r="AI15" s="56">
+        <v>37960</v>
+      </c>
+      <c r="AJ15" s="56">
+        <v>41960</v>
+      </c>
+      <c r="AR15" s="56">
+        <v>17800</v>
+      </c>
+      <c r="AS15" s="56">
+        <v>19700</v>
+      </c>
+      <c r="AT15" s="56">
+        <v>21400</v>
+      </c>
+      <c r="AU15" s="56">
+        <v>25500</v>
+      </c>
+      <c r="AV15" s="56">
+        <v>32660</v>
+      </c>
+      <c r="AW15" s="56">
+        <v>36860</v>
+      </c>
+      <c r="AX15" s="56">
+        <v>40860</v>
+      </c>
+      <c r="BF15" s="56">
+        <v>52780</v>
+      </c>
+      <c r="BG15" s="56">
+        <v>71780</v>
+      </c>
+      <c r="BH15" s="56">
+        <v>87180</v>
+      </c>
+      <c r="BI15" s="56">
+        <v>99180</v>
+      </c>
+      <c r="BJ15" s="56">
+        <v>41780</v>
+      </c>
+      <c r="BK15" s="56">
+        <v>74780</v>
+      </c>
+      <c r="BL15" s="56">
+        <v>115000</v>
+      </c>
+      <c r="BM15" s="56">
+        <v>131000</v>
+      </c>
+      <c r="BN15" s="56">
+        <v>147000</v>
+      </c>
+      <c r="BO15" s="56">
+        <v>188000</v>
+      </c>
+      <c r="BP15" s="56">
+        <v>282000</v>
+      </c>
+      <c r="BQ15" s="56">
+        <v>330000</v>
+      </c>
+      <c r="BR15" s="56">
+        <v>190000</v>
+      </c>
+      <c r="BS15" s="56">
+        <v>219000</v>
+      </c>
+      <c r="BT15" s="56">
+        <v>173000</v>
+      </c>
+      <c r="BU15" s="56">
+        <v>197000</v>
+      </c>
+      <c r="BV15" s="56">
+        <v>224000</v>
+      </c>
+      <c r="BW15" s="56">
+        <v>110500</v>
+      </c>
+      <c r="BX15" s="56">
+        <v>125800</v>
+      </c>
+      <c r="BY15" s="56">
+        <v>141100</v>
+      </c>
+      <c r="BZ15" s="56">
+        <v>235600</v>
+      </c>
+      <c r="CA15" s="56">
+        <v>28900</v>
+      </c>
+      <c r="CB15" s="56">
+        <v>33900</v>
+      </c>
+      <c r="CC15" s="56">
+        <v>390500</v>
+      </c>
+      <c r="CD15" s="56">
+        <v>443500</v>
+      </c>
+      <c r="CE15" s="56">
+        <v>497500</v>
+      </c>
+      <c r="CF15" s="56">
+        <v>547300</v>
+      </c>
+      <c r="CG15" s="56">
+        <v>628000</v>
+      </c>
+      <c r="CH15" s="56">
+        <v>678000</v>
+      </c>
+      <c r="CI15" s="56">
+        <v>729500</v>
+      </c>
+      <c r="CJ15" s="56">
+        <v>782500</v>
+      </c>
+      <c r="CK15" s="56">
+        <v>834000</v>
+      </c>
+      <c r="CL15" s="56">
+        <v>888000</v>
+      </c>
+      <c r="CM15" s="56">
+        <v>941000</v>
+      </c>
+      <c r="CN15" s="56">
+        <v>995000</v>
+      </c>
+      <c r="CO15" s="56">
+        <v>1044800</v>
+      </c>
+      <c r="CP15" s="56">
+        <v>1094600</v>
+      </c>
+      <c r="CQ15" s="56">
+        <v>1175500</v>
+      </c>
+      <c r="CR15" s="56">
+        <v>1225300</v>
+      </c>
+      <c r="CS15" s="56">
+        <v>1278500</v>
+      </c>
+      <c r="CT15" s="56">
+        <v>1331500</v>
+      </c>
+      <c r="CU15" s="56">
+        <v>1385500</v>
+      </c>
+      <c r="CV15" s="56">
+        <v>1438500</v>
+      </c>
+      <c r="CW15" s="56">
+        <v>1492500</v>
+      </c>
+      <c r="CX15" s="56">
+        <v>1542300</v>
+      </c>
+      <c r="CY15" s="56">
+        <v>1592100</v>
+      </c>
+      <c r="CZ15" s="56">
+        <v>1641900</v>
+      </c>
+      <c r="DA15" s="56">
+        <v>282000</v>
+      </c>
+      <c r="DB15" s="56">
+        <v>346000</v>
+      </c>
+      <c r="DC15" s="56">
+        <v>406000</v>
+      </c>
+      <c r="DD15" s="56">
+        <v>469500</v>
+      </c>
+      <c r="DE15" s="56">
+        <v>529500</v>
+      </c>
+      <c r="DF15" s="56">
+        <v>595500</v>
+      </c>
+      <c r="DG15" s="56">
+        <v>655300</v>
+      </c>
+      <c r="DH15" s="56">
+        <v>752000</v>
+      </c>
+      <c r="DI15" s="56">
+        <v>812000</v>
+      </c>
+      <c r="DJ15" s="56">
+        <v>875500</v>
+      </c>
+      <c r="DK15" s="56">
+        <v>935500</v>
+      </c>
+      <c r="DL15" s="56">
+        <v>999000</v>
+      </c>
+      <c r="DM15" s="56">
+        <v>1065000</v>
+      </c>
+      <c r="DN15" s="56">
+        <v>1125000</v>
+      </c>
+      <c r="DO15" s="56">
+        <v>1191000</v>
+      </c>
+      <c r="DP15" s="56">
+        <v>1250800</v>
+      </c>
+      <c r="DQ15" s="56">
+        <v>1310600</v>
+      </c>
+      <c r="DR15" s="56">
+        <v>1407500</v>
+      </c>
+      <c r="DS15" s="56">
+        <v>1467300</v>
+      </c>
+      <c r="DT15" s="56">
+        <v>1534500</v>
+      </c>
+      <c r="DU15" s="56">
+        <v>1594500</v>
+      </c>
+      <c r="DV15" s="56">
+        <v>1660500</v>
+      </c>
+      <c r="DW15" s="56">
+        <v>1720500</v>
+      </c>
+      <c r="DX15" s="56">
+        <v>1786500</v>
+      </c>
+      <c r="DY15" s="56">
+        <v>1846300</v>
+      </c>
+      <c r="DZ15" s="56">
+        <v>1906100</v>
+      </c>
+      <c r="EA15" s="56">
+        <v>1965900</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -16264,7 +18067,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB764343-28B8-406D-977B-66BB2AAB408D}">
   <dimension ref="A1:AF19"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -17792,7 +19595,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{416E1F1A-25CB-4357-AA92-79D3362290DE}">
   <dimension ref="A1:BL17"/>
   <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
feat: release v2.18.0 - VRV indoor prefix, horizontal piping diagram, remove notice box, and aggregate quotation equipment
</commit_message>
<xml_diff>
--- a/backend/product_database/EQUIPMENT_Data.xlsx
+++ b/backend/product_database/EQUIPMENT_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flitt\.gemini\antigravity\scratch\ac-selection-system\backend\product_database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0462C98F-FDE6-4E9D-B2C0-7C240F28F3B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB331C89-B0CA-40D5-A8AB-19BD2169064E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="324" yWindow="120" windowWidth="15504" windowHeight="12240" activeTab="1" xr2:uid="{B9AE4098-F0A1-4C76-B9D5-37F1BE2208A4}"/>
+    <workbookView xWindow="324" yWindow="120" windowWidth="17640" windowHeight="12240" activeTab="1" xr2:uid="{B9AE4098-F0A1-4C76-B9D5-37F1BE2208A4}"/>
   </bookViews>
   <sheets>
     <sheet name="indoor_units" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3780" uniqueCount="623">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3784" uniqueCount="623">
   <si>
     <t>資料型態</t>
   </si>
@@ -12121,7 +12121,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F00506A-09F5-4009-80F2-281B4A4C3425}">
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
@@ -12132,9 +12132,10 @@
     <col min="9" max="9" width="12.88671875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.44140625" customWidth="1"/>
     <col min="12" max="12" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>569</v>
       </c>
@@ -12147,8 +12148,11 @@
       <c r="L1" t="s">
         <v>612</v>
       </c>
+      <c r="O1" t="s">
+        <v>557</v>
+      </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>605</v>
       </c>
@@ -12179,8 +12183,14 @@
       <c r="M2" t="s">
         <v>607</v>
       </c>
+      <c r="O2" t="s">
+        <v>605</v>
+      </c>
+      <c r="P2" t="s">
+        <v>607</v>
+      </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="61" t="s">
         <v>570</v>
       </c>
@@ -12211,8 +12221,11 @@
       <c r="M3">
         <v>4500</v>
       </c>
+      <c r="O3" t="s">
+        <v>561</v>
+      </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="61" t="s">
         <v>573</v>
       </c>
@@ -12238,7 +12251,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>581</v>
       </c>
@@ -12255,7 +12268,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="61" t="s">
         <v>574</v>
       </c>
@@ -12269,7 +12282,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>575</v>
       </c>
@@ -12280,7 +12293,7 @@
         <v>7350</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="61" t="s">
         <v>578</v>
       </c>
@@ -12294,7 +12307,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>579</v>
       </c>
@@ -12305,7 +12318,7 @@
         <v>2800</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="61" t="s">
         <v>584</v>
       </c>
@@ -12320,7 +12333,7 @@
       </c>
       <c r="F10" s="62"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>586</v>
       </c>
@@ -12331,7 +12344,7 @@
         <v>28600</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>588</v>
       </c>
@@ -12342,7 +12355,7 @@
         <v>19400</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>591</v>
       </c>
@@ -12356,7 +12369,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>590</v>
       </c>
@@ -12367,7 +12380,7 @@
         <v>27500</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" s="61" t="s">
         <v>594</v>
       </c>
@@ -12381,7 +12394,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" s="61" t="s">
         <v>598</v>
       </c>

</xml_diff>

<commit_message>
feat: release v2.19.0 - add remove space option to table context menu
</commit_message>
<xml_diff>
--- a/backend/product_database/EQUIPMENT_Data.xlsx
+++ b/backend/product_database/EQUIPMENT_Data.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flitt\.gemini\antigravity\scratch\ac-selection-system\backend\product_database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB331C89-B0CA-40D5-A8AB-19BD2169064E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB112E35-1FDE-4E0D-97F1-D9D2A82C0CE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="324" yWindow="120" windowWidth="17640" windowHeight="12240" activeTab="1" xr2:uid="{B9AE4098-F0A1-4C76-B9D5-37F1BE2208A4}"/>
   </bookViews>
   <sheets>
     <sheet name="indoor_units" sheetId="1" r:id="rId1"/>
-    <sheet name="controller" sheetId="5" r:id="rId2"/>
+    <sheet name="controller&amp;pipe" sheetId="5" r:id="rId2"/>
     <sheet name="outdoor_units" sheetId="2" r:id="rId3"/>
     <sheet name="indoor_units_SA only" sheetId="3" r:id="rId4"/>
     <sheet name="outdoor_units_SA only" sheetId="4" r:id="rId5"/>

</xml_diff>

<commit_message>
feat: release v2.19.0 - scale cursor precision alignment, controller&pipe accessory pricing, and VRV Table 5 / SA pipe sizing
</commit_message>
<xml_diff>
--- a/backend/product_database/EQUIPMENT_Data.xlsx
+++ b/backend/product_database/EQUIPMENT_Data.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flitt\.gemini\antigravity\scratch\ac-selection-system\backend\product_database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB331C89-B0CA-40D5-A8AB-19BD2169064E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DB81D03-8E0B-48F4-8387-5337B7480ABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="324" yWindow="120" windowWidth="17640" windowHeight="12240" activeTab="1" xr2:uid="{B9AE4098-F0A1-4C76-B9D5-37F1BE2208A4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{B9AE4098-F0A1-4C76-B9D5-37F1BE2208A4}"/>
   </bookViews>
   <sheets>
     <sheet name="indoor_units" sheetId="1" r:id="rId1"/>
-    <sheet name="controller" sheetId="5" r:id="rId2"/>
+    <sheet name="controller&amp;pipe" sheetId="5" r:id="rId2"/>
     <sheet name="outdoor_units" sheetId="2" r:id="rId3"/>
     <sheet name="indoor_units_SA only" sheetId="3" r:id="rId4"/>
     <sheet name="outdoor_units_SA only" sheetId="4" r:id="rId5"/>
@@ -12224,6 +12224,9 @@
       <c r="O3" t="s">
         <v>561</v>
       </c>
+      <c r="P3">
+        <v>4300</v>
+      </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="61" t="s">

</xml_diff>

<commit_message>
fix: sync outdoor model in piping diagram dropdown, restore missing joints in system sheet, fix nominal cap & power consumption export, and update HRV pricing with PM2.5 filter & remote
</commit_message>
<xml_diff>
--- a/backend/product_database/EQUIPMENT_Data.xlsx
+++ b/backend/product_database/EQUIPMENT_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flitt\.gemini\antigravity\scratch\ac-selection-system\backend\product_database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{563775CE-1ECE-40EA-999D-9C9764F8B12F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB8C6114-3219-413E-A454-5D1A9240C7A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2028" yWindow="2088" windowWidth="17640" windowHeight="9444" firstSheet="3" activeTab="5" xr2:uid="{B9AE4098-F0A1-4C76-B9D5-37F1BE2208A4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="5" xr2:uid="{B9AE4098-F0A1-4C76-B9D5-37F1BE2208A4}"/>
   </bookViews>
   <sheets>
     <sheet name="indoor_units" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3863" uniqueCount="653">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3866" uniqueCount="660">
   <si>
     <t>資料型態</t>
   </si>
@@ -2516,6 +2516,34 @@
   </si>
   <si>
     <t>785×1,012×1,110</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PM2.5濾網價格(NT$)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BAFH510A250</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BAFH510A350</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BAFH510A650</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BAFH510A2000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BAFH510A2000+BAFH510A2000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BRC1H63W</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2631,7 +2659,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -2732,13 +2760,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2939,6 +2980,18 @@
     </xf>
     <xf numFmtId="177" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -12406,6 +12459,12 @@
       <c r="J4">
         <v>1600</v>
       </c>
+      <c r="O4" t="s">
+        <v>659</v>
+      </c>
+      <c r="P4">
+        <v>4000</v>
+      </c>
       <c r="R4" t="s">
         <v>628</v>
       </c>
@@ -22009,7 +22068,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="65" t="s">
         <v>646</v>
       </c>
@@ -22019,31 +22078,31 @@
       <c r="C5" s="65"/>
       <c r="D5" s="65"/>
       <c r="E5" s="12" t="s">
-        <v>536</v>
+        <v>654</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>536</v>
+        <v>654</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>536</v>
+        <v>655</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>536</v>
+        <v>656</v>
       </c>
       <c r="I5" s="12" t="s">
-        <v>536</v>
+        <v>656</v>
       </c>
       <c r="J5" s="12" t="s">
-        <v>536</v>
+        <v>657</v>
       </c>
       <c r="K5" s="12" t="s">
-        <v>536</v>
-      </c>
-      <c r="L5" s="12" t="s">
-        <v>536</v>
-      </c>
-      <c r="M5" s="12" t="s">
-        <v>536</v>
+        <v>657</v>
+      </c>
+      <c r="L5" s="67" t="s">
+        <v>658</v>
+      </c>
+      <c r="M5" s="67" t="s">
+        <v>658</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
@@ -22083,48 +22142,48 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="65" t="s">
+    <row r="7" spans="1:13" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="68" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="65" t="s">
+      <c r="B7" s="68" t="s">
         <v>60</v>
       </c>
-      <c r="C7" s="65"/>
-      <c r="D7" s="65"/>
-      <c r="E7" s="12">
+      <c r="C7" s="68"/>
+      <c r="D7" s="68"/>
+      <c r="E7" s="69">
         <f>0.03*2</f>
         <v>0.06</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="69">
         <f>0.03*2</f>
         <v>0.06</v>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="69">
         <f>0.06*2</f>
         <v>0.12</v>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="69">
         <f>0.1*2</f>
         <v>0.2</v>
       </c>
-      <c r="I7" s="12">
+      <c r="I7" s="69">
         <f>0.17*2</f>
         <v>0.34</v>
       </c>
-      <c r="J7" s="12">
+      <c r="J7" s="69">
         <f>0.19*2</f>
         <v>0.38</v>
       </c>
-      <c r="K7" s="12">
+      <c r="K7" s="69">
         <f>0.19*2</f>
         <v>0.38</v>
       </c>
-      <c r="L7" s="12">
+      <c r="L7" s="69">
         <f>0.19*4</f>
         <v>0.76</v>
       </c>
-      <c r="M7" s="12">
+      <c r="M7" s="69">
         <f>0.19*4</f>
         <v>0.76</v>
       </c>
@@ -22138,31 +22197,31 @@
       </c>
       <c r="C8" s="65"/>
       <c r="D8" s="65"/>
-      <c r="E8" s="15" t="s">
+      <c r="E8" s="64" t="s">
         <v>648</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="64" t="s">
         <v>648</v>
       </c>
-      <c r="G8" s="15" t="s">
+      <c r="G8" s="64" t="s">
         <v>649</v>
       </c>
-      <c r="H8" s="15" t="s">
+      <c r="H8" s="64" t="s">
         <v>650</v>
       </c>
-      <c r="I8" s="15" t="s">
+      <c r="I8" s="64" t="s">
         <v>650</v>
       </c>
-      <c r="J8" s="15" t="s">
+      <c r="J8" s="64" t="s">
         <v>651</v>
       </c>
-      <c r="K8" s="15" t="s">
+      <c r="K8" s="64" t="s">
         <v>651</v>
       </c>
-      <c r="L8" s="15" t="s">
+      <c r="L8" s="64" t="s">
         <v>652</v>
       </c>
-      <c r="M8" s="15" t="s">
+      <c r="M8" s="64" t="s">
         <v>652</v>
       </c>
     </row>
@@ -22175,36 +22234,72 @@
       </c>
       <c r="C9" s="66"/>
       <c r="D9" s="66"/>
-      <c r="E9" s="49">
-        <v>50000</v>
-      </c>
-      <c r="F9" s="49">
-        <v>60000</v>
-      </c>
-      <c r="G9" s="49">
-        <v>70000</v>
-      </c>
-      <c r="H9" s="49">
-        <v>80000</v>
-      </c>
-      <c r="I9" s="49">
-        <v>50000</v>
-      </c>
-      <c r="J9" s="49">
-        <v>50000</v>
-      </c>
-      <c r="K9" s="49">
-        <v>50000</v>
-      </c>
-      <c r="L9" s="49">
-        <v>50000</v>
-      </c>
-      <c r="M9" s="49">
-        <v>50000</v>
+      <c r="E9" s="70">
+        <v>34600</v>
+      </c>
+      <c r="F9" s="70">
+        <v>36800</v>
+      </c>
+      <c r="G9" s="70">
+        <v>42700</v>
+      </c>
+      <c r="H9" s="70">
+        <v>45800</v>
+      </c>
+      <c r="I9" s="70">
+        <v>51800</v>
+      </c>
+      <c r="J9" s="70">
+        <v>69100</v>
+      </c>
+      <c r="K9" s="70">
+        <v>81300</v>
+      </c>
+      <c r="L9" s="70">
+        <v>122700</v>
+      </c>
+      <c r="M9" s="70">
+        <v>150000</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A10" s="24"/>
+    <row r="10" spans="1:13" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="17" t="s">
+        <v>653</v>
+      </c>
+      <c r="B10" s="65" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="70">
+        <v>2500</v>
+      </c>
+      <c r="F10" s="70">
+        <v>2500</v>
+      </c>
+      <c r="G10" s="70">
+        <v>3200</v>
+      </c>
+      <c r="H10" s="70">
+        <v>5500</v>
+      </c>
+      <c r="I10" s="70">
+        <v>5500</v>
+      </c>
+      <c r="J10" s="70">
+        <v>6500</v>
+      </c>
+      <c r="K10" s="70">
+        <v>6500</v>
+      </c>
+      <c r="L10" s="70">
+        <f>6500*2</f>
+        <v>13000</v>
+      </c>
+      <c r="M10" s="70">
+        <f>6500*2</f>
+        <v>13000</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>